<commit_message>
fix: proper number formatting, stipend reframe, INR header
Number formatting:
- New _num_fmt() helper: ints get '#,##0', decimals get '#,##0.##'
- Applied per-cell to cols E (qty), F (unit cost), G (total cost)
- Whole-number floats auto-cast to int before writing to cell
- Total Cost col G always uses '#,##0' (formula results are ints)

Stipends reframed (all 4 phases):
- qty=5 (people), unit=12,500 (half-month rate per person)
- Specs: '5 students x 2 weeks (0.5 month) @ Rs. 25,000/person/month'
- Notes: 'Rs. 25,000/person/month x 0.5 month x 5 students = Rs. 62,500'
- Total via =E*F = 62,500 (unchanged)

Header: added '| All prices in INR'

Verified: zero formula errors, all subtotals correct
</commit_message>
<xml_diff>
--- a/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
+++ b/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Delhi-PS-CRM\QuotationSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5FA4E0-7611-434C-86D9-F580833105EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785ACB68-A2AA-4CD1-8F49-1541300D42EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="166">
   <si>
     <t>Delhi PS-CRM — Project Cost Quotation</t>
   </si>
@@ -42,7 +42,7 @@
     <t>AI-Powered WhatsApp Civic Complaint Management System</t>
   </si>
   <si>
-    <t>Team: Delhi PS-CRM | Document: Cost Quotation v2.0 | Excluding all applicable taxes</t>
+    <t>Team: Delhi PS-CRM | Document: Cost Quotation v2.0 | Excluding all applicable taxes | All prices in INR</t>
   </si>
   <si>
     <t>SECTION 1 — PROJECT OVERVIEW HEADER</t>
@@ -201,10 +201,10 @@
     <t>Student Developer Stipends</t>
   </si>
   <si>
-    <t>5 team members: backend, ML integration, architecture, testing, DevOps</t>
-  </si>
-  <si>
-    <t>Half-month stipend weeks 1-2</t>
+    <t>5 students × 2 weeks (0.5 month) @ Rs. 25,000/person/month</t>
+  </si>
+  <si>
+    <t>Rs. 25,000/person/month × 0.5 month × 5 students = Rs. 62,500</t>
   </si>
   <si>
     <t>Infrastructure</t>
@@ -261,12 +261,6 @@
     <t>Phase 1 Subtotal</t>
   </si>
   <si>
-    <t>5 members during pilot: monitoring, bug fixes, officer onboarding</t>
-  </si>
-  <si>
-    <t>Half-month stipend weeks 3-4</t>
-  </si>
-  <si>
     <t>Azure Container Apps</t>
   </si>
   <si>
@@ -330,12 +324,6 @@
     <t>Phase 2 Subtotal</t>
   </si>
   <si>
-    <t>Scaling support, QA, officer training, data ops</t>
-  </si>
-  <si>
-    <t>Half-month stipend weeks 5-6</t>
-  </si>
-  <si>
     <t>Scaled backend for 50 wards</t>
   </si>
   <si>
@@ -415,12 +403,6 @@
   </si>
   <si>
     <t>Phase 3 Subtotal</t>
-  </si>
-  <si>
-    <t>Full-scale deployment support, ward onboarding, stress testing</t>
-  </si>
-  <si>
-    <t>Half-month stipend weeks 7-8</t>
   </si>
   <si>
     <t>Full-scale auto-scaling for 272 wards</t>
@@ -556,10 +538,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.##"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.##"/>
     <numFmt numFmtId="165" formatCode="###,##0"/>
-    <numFmt numFmtId="166" formatCode="0.00#"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -801,7 +782,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -842,34 +823,28 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="7" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -1260,118 +1235,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="52" t="s">
+      <c r="A6" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="54" t="s">
+      <c r="B6" s="33"/>
+      <c r="C6" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="36"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="34"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="54" t="s">
+      <c r="B7" s="33"/>
+      <c r="C7" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="36"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="54" t="s">
+      <c r="B8" s="33"/>
+      <c r="C8" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="38"/>
-      <c r="C9" s="37" t="s">
+      <c r="B9" s="36"/>
+      <c r="C9" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="39"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="37"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="45"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="43"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -1499,42 +1474,42 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="12">
         <f>G30+G38+G50+G62</f>
         <v>322758</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="57" t="s">
+      <c r="A20" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
       <c r="F20" s="13">
         <f>G75*12</f>
         <v>676680</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="44"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="45"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="43"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
@@ -1576,17 +1551,16 @@
         <v>55</v>
       </c>
       <c r="E24" s="14">
-        <f>5*0.5</f>
-        <v>2.5</v>
-      </c>
-      <c r="F24" s="15">
-        <v>25000</v>
-      </c>
-      <c r="G24" s="15">
+        <v>5</v>
+      </c>
+      <c r="F24" s="14">
+        <v>12500</v>
+      </c>
+      <c r="G24" s="14">
         <f t="shared" ref="G24:G29" si="0">E24*F24</f>
         <v>62500</v>
       </c>
-      <c r="H24" s="16" t="s">
+      <c r="H24" s="15" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1603,17 +1577,17 @@
       <c r="D25" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="17">
+      <c r="E25" s="16">
         <v>0.5</v>
       </c>
-      <c r="F25" s="18">
+      <c r="F25" s="17">
         <v>4000</v>
       </c>
-      <c r="G25" s="18">
+      <c r="G25" s="17">
         <f t="shared" si="0"/>
         <v>2000</v>
       </c>
-      <c r="H25" s="19" t="s">
+      <c r="H25" s="18" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1630,17 +1604,17 @@
       <c r="D26" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="14">
+      <c r="E26" s="19">
         <v>0.5</v>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="14">
         <v>2500</v>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="14">
         <f t="shared" si="0"/>
         <v>1250</v>
       </c>
-      <c r="H26" s="16" t="s">
+      <c r="H26" s="15" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1660,14 +1634,14 @@
       <c r="E27" s="17">
         <v>1</v>
       </c>
-      <c r="F27" s="18">
+      <c r="F27" s="17">
         <v>5000</v>
       </c>
-      <c r="G27" s="18">
+      <c r="G27" s="17">
         <f t="shared" si="0"/>
         <v>5000</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="18" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1687,14 +1661,14 @@
       <c r="E28" s="14">
         <v>1</v>
       </c>
-      <c r="F28" s="15">
+      <c r="F28" s="14">
         <v>4000</v>
       </c>
-      <c r="G28" s="15">
+      <c r="G28" s="14">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
-      <c r="H28" s="16" t="s">
+      <c r="H28" s="15" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1714,26 +1688,26 @@
       <c r="E29" s="17">
         <v>1</v>
       </c>
-      <c r="F29" s="18">
+      <c r="F29" s="17">
         <v>1000</v>
       </c>
-      <c r="G29" s="18">
+      <c r="G29" s="17">
         <f t="shared" si="0"/>
         <v>1000</v>
       </c>
-      <c r="H29" s="19" t="s">
+      <c r="H29" s="18" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="46" t="s">
+      <c r="A30" s="44" t="s">
         <v>74</v>
       </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
       <c r="G30" s="20">
         <f>SUM(G24:G29)</f>
         <v>75750</v>
@@ -1751,21 +1725,20 @@
         <v>54</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E31" s="14">
-        <f>5*0.5</f>
-        <v>2.5</v>
-      </c>
-      <c r="F31" s="15">
-        <v>25000</v>
-      </c>
-      <c r="G31" s="15">
+        <v>5</v>
+      </c>
+      <c r="F31" s="14">
+        <v>12500</v>
+      </c>
+      <c r="G31" s="14">
         <f t="shared" ref="G31:G37" si="1">E31*F31</f>
         <v>62500</v>
       </c>
-      <c r="H31" s="16" t="s">
-        <v>76</v>
+      <c r="H31" s="15" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
@@ -1776,23 +1749,23 @@
         <v>57</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="17">
+        <v>76</v>
+      </c>
+      <c r="E32" s="16">
         <v>0.5</v>
       </c>
-      <c r="F32" s="18">
+      <c r="F32" s="17">
         <v>4000</v>
       </c>
-      <c r="G32" s="18">
+      <c r="G32" s="17">
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="H32" s="19" t="s">
-        <v>79</v>
+      <c r="H32" s="18" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
@@ -1803,23 +1776,23 @@
         <v>57</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E33" s="14">
+        <v>79</v>
+      </c>
+      <c r="E33" s="19">
         <v>0.5</v>
       </c>
-      <c r="F33" s="15">
+      <c r="F33" s="14">
         <v>2500</v>
       </c>
-      <c r="G33" s="15">
+      <c r="G33" s="14">
         <f t="shared" si="1"/>
         <v>1250</v>
       </c>
-      <c r="H33" s="16" t="s">
-        <v>82</v>
+      <c r="H33" s="15" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
@@ -1830,23 +1803,23 @@
         <v>57</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E34" s="17">
+        <v>82</v>
+      </c>
+      <c r="E34" s="16">
         <v>0.5</v>
       </c>
-      <c r="F34" s="18">
+      <c r="F34" s="17">
         <v>500</v>
       </c>
-      <c r="G34" s="18">
+      <c r="G34" s="17">
         <f t="shared" si="1"/>
         <v>250</v>
       </c>
-      <c r="H34" s="19" t="s">
-        <v>85</v>
+      <c r="H34" s="18" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
@@ -1854,26 +1827,26 @@
         <v>24</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="E35" s="14">
         <v>1000</v>
       </c>
-      <c r="F35" s="22">
+      <c r="F35" s="19">
         <v>0.05</v>
       </c>
-      <c r="G35" s="15">
+      <c r="G35" s="14">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="H35" s="16" t="s">
-        <v>89</v>
+      <c r="H35" s="15" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -1881,26 +1854,26 @@
         <v>24</v>
       </c>
       <c r="B36" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D36" s="9" t="s">
         <v>90</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>92</v>
       </c>
       <c r="E36" s="17">
         <v>1000</v>
       </c>
-      <c r="F36" s="23">
+      <c r="F36" s="16">
         <v>0.1</v>
       </c>
-      <c r="G36" s="18">
+      <c r="G36" s="17">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="H36" s="19" t="s">
-        <v>93</v>
+      <c r="H36" s="18" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
@@ -1908,37 +1881,37 @@
         <v>24</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E37" s="14">
         <v>1</v>
       </c>
-      <c r="F37" s="15">
+      <c r="F37" s="14">
         <v>100</v>
       </c>
-      <c r="G37" s="15">
+      <c r="G37" s="14">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="H37" s="16" t="s">
-        <v>96</v>
+      <c r="H37" s="15" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="46" t="s">
-        <v>97</v>
-      </c>
-      <c r="B38" s="35"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="35"/>
+      <c r="A38" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="33"/>
+      <c r="C38" s="33"/>
+      <c r="D38" s="33"/>
+      <c r="E38" s="33"/>
+      <c r="F38" s="33"/>
       <c r="G38" s="20">
         <f>SUM(G31:G37)</f>
         <v>66250</v>
@@ -1956,21 +1929,20 @@
         <v>54</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>98</v>
+        <v>55</v>
       </c>
       <c r="E39" s="17">
-        <f>5*0.5</f>
-        <v>2.5</v>
-      </c>
-      <c r="F39" s="18">
-        <v>25000</v>
-      </c>
-      <c r="G39" s="18">
+        <v>5</v>
+      </c>
+      <c r="F39" s="17">
+        <v>12500</v>
+      </c>
+      <c r="G39" s="17">
         <f t="shared" ref="G39:G49" si="2">E39*F39</f>
         <v>62500</v>
       </c>
-      <c r="H39" s="19" t="s">
-        <v>99</v>
+      <c r="H39" s="18" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
@@ -1981,23 +1953,23 @@
         <v>57</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E40" s="14">
+        <v>96</v>
+      </c>
+      <c r="E40" s="19">
         <v>0.5</v>
       </c>
-      <c r="F40" s="15">
+      <c r="F40" s="14">
         <v>8000</v>
       </c>
-      <c r="G40" s="15">
+      <c r="G40" s="14">
         <f t="shared" si="2"/>
         <v>4000</v>
       </c>
-      <c r="H40" s="16" t="s">
-        <v>101</v>
+      <c r="H40" s="15" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
@@ -2008,23 +1980,23 @@
         <v>57</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="E41" s="17">
+        <v>99</v>
+      </c>
+      <c r="E41" s="16">
         <v>0.5</v>
       </c>
-      <c r="F41" s="18">
+      <c r="F41" s="17">
         <v>5000</v>
       </c>
-      <c r="G41" s="18">
+      <c r="G41" s="17">
         <f t="shared" si="2"/>
         <v>2500</v>
       </c>
-      <c r="H41" s="19" t="s">
-        <v>104</v>
+      <c r="H41" s="18" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
@@ -2035,23 +2007,23 @@
         <v>57</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E42" s="14">
+        <v>101</v>
+      </c>
+      <c r="E42" s="19">
         <v>0.5</v>
       </c>
-      <c r="F42" s="15">
+      <c r="F42" s="14">
         <v>1500</v>
       </c>
-      <c r="G42" s="15">
+      <c r="G42" s="14">
         <f t="shared" si="2"/>
         <v>750</v>
       </c>
-      <c r="H42" s="16" t="s">
-        <v>106</v>
+      <c r="H42" s="15" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
@@ -2062,23 +2034,23 @@
         <v>57</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="E43" s="17">
+        <v>104</v>
+      </c>
+      <c r="E43" s="16">
         <v>0.5</v>
       </c>
-      <c r="F43" s="18">
+      <c r="F43" s="17">
         <v>1500</v>
       </c>
-      <c r="G43" s="18">
+      <c r="G43" s="17">
         <f t="shared" si="2"/>
         <v>750</v>
       </c>
-      <c r="H43" s="19" t="s">
-        <v>109</v>
+      <c r="H43" s="18" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
@@ -2089,23 +2061,23 @@
         <v>57</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E44" s="14">
+        <v>107</v>
+      </c>
+      <c r="E44" s="19">
         <v>0.5</v>
       </c>
-      <c r="F44" s="15">
+      <c r="F44" s="14">
         <v>1000</v>
       </c>
-      <c r="G44" s="15">
+      <c r="G44" s="14">
         <f t="shared" si="2"/>
         <v>500</v>
       </c>
-      <c r="H44" s="16" t="s">
-        <v>112</v>
+      <c r="H44" s="15" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
@@ -2113,26 +2085,26 @@
         <v>29</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E45" s="17">
         <v>20000</v>
       </c>
-      <c r="F45" s="23">
+      <c r="F45" s="16">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="G45" s="18">
+      <c r="G45" s="17">
         <f t="shared" si="2"/>
         <v>300</v>
       </c>
-      <c r="H45" s="19" t="s">
-        <v>114</v>
+      <c r="H45" s="18" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
@@ -2140,26 +2112,26 @@
         <v>29</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E46" s="14">
         <v>1</v>
       </c>
-      <c r="F46" s="15">
+      <c r="F46" s="14">
         <v>8000</v>
       </c>
-      <c r="G46" s="15">
+      <c r="G46" s="14">
         <f t="shared" si="2"/>
         <v>8000</v>
       </c>
-      <c r="H46" s="16" t="s">
-        <v>117</v>
+      <c r="H46" s="15" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
@@ -2167,26 +2139,26 @@
         <v>29</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E47" s="17">
         <v>20000</v>
       </c>
-      <c r="F47" s="23">
+      <c r="F47" s="16">
         <v>0.06</v>
       </c>
-      <c r="G47" s="18">
+      <c r="G47" s="17">
         <f t="shared" si="2"/>
         <v>1200</v>
       </c>
-      <c r="H47" s="19" t="s">
-        <v>119</v>
+      <c r="H47" s="18" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
@@ -2194,26 +2166,26 @@
         <v>29</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="E48" s="14">
+        <v>117</v>
+      </c>
+      <c r="E48" s="19">
         <v>0.5</v>
       </c>
-      <c r="F48" s="15">
+      <c r="F48" s="14">
         <v>1676</v>
       </c>
-      <c r="G48" s="15">
+      <c r="G48" s="14">
         <f t="shared" si="2"/>
         <v>838</v>
       </c>
-      <c r="H48" s="16" t="s">
-        <v>122</v>
+      <c r="H48" s="15" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
@@ -2224,34 +2196,34 @@
         <v>57</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="E49" s="17">
+        <v>120</v>
+      </c>
+      <c r="E49" s="16">
         <v>0.5</v>
       </c>
-      <c r="F49" s="18">
+      <c r="F49" s="17">
         <v>1500</v>
       </c>
-      <c r="G49" s="18">
+      <c r="G49" s="17">
         <f t="shared" si="2"/>
         <v>750</v>
       </c>
-      <c r="H49" s="19" t="s">
-        <v>125</v>
+      <c r="H49" s="18" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="46" t="s">
-        <v>126</v>
-      </c>
-      <c r="B50" s="35"/>
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="35"/>
-      <c r="F50" s="35"/>
+      <c r="A50" s="44" t="s">
+        <v>122</v>
+      </c>
+      <c r="B50" s="33"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="33"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="33"/>
       <c r="G50" s="20">
         <f>SUM(G39:G49)</f>
         <v>82088</v>
@@ -2269,21 +2241,20 @@
         <v>54</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>127</v>
+        <v>55</v>
       </c>
       <c r="E51" s="14">
-        <f>5*0.5</f>
-        <v>2.5</v>
-      </c>
-      <c r="F51" s="15">
-        <v>25000</v>
-      </c>
-      <c r="G51" s="15">
+        <v>5</v>
+      </c>
+      <c r="F51" s="14">
+        <v>12500</v>
+      </c>
+      <c r="G51" s="14">
         <f t="shared" ref="G51:G61" si="3">E51*F51</f>
         <v>62500</v>
       </c>
-      <c r="H51" s="16" t="s">
-        <v>128</v>
+      <c r="H51" s="15" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
@@ -2294,23 +2265,23 @@
         <v>57</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="E52" s="17">
+        <v>123</v>
+      </c>
+      <c r="E52" s="16">
         <v>0.5</v>
       </c>
-      <c r="F52" s="18">
+      <c r="F52" s="17">
         <v>15000</v>
       </c>
-      <c r="G52" s="18">
+      <c r="G52" s="17">
         <f t="shared" si="3"/>
         <v>7500</v>
       </c>
-      <c r="H52" s="19" t="s">
-        <v>130</v>
+      <c r="H52" s="18" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2321,23 +2292,23 @@
         <v>57</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="E53" s="14">
+        <v>125</v>
+      </c>
+      <c r="E53" s="19">
         <v>0.5</v>
       </c>
-      <c r="F53" s="15">
+      <c r="F53" s="14">
         <v>12000</v>
       </c>
-      <c r="G53" s="15">
+      <c r="G53" s="14">
         <f t="shared" si="3"/>
         <v>6000</v>
       </c>
-      <c r="H53" s="16" t="s">
-        <v>132</v>
+      <c r="H53" s="15" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
@@ -2348,23 +2319,23 @@
         <v>57</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E54" s="17">
+        <v>127</v>
+      </c>
+      <c r="E54" s="16">
         <v>0.5</v>
       </c>
-      <c r="F54" s="18">
+      <c r="F54" s="17">
         <v>4000</v>
       </c>
-      <c r="G54" s="18">
+      <c r="G54" s="17">
         <f t="shared" si="3"/>
         <v>2000</v>
       </c>
-      <c r="H54" s="19" t="s">
-        <v>134</v>
+      <c r="H54" s="18" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
@@ -2375,23 +2346,23 @@
         <v>57</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E55" s="14">
+        <v>129</v>
+      </c>
+      <c r="E55" s="19">
         <v>0.5</v>
       </c>
-      <c r="F55" s="15">
+      <c r="F55" s="14">
         <v>3000</v>
       </c>
-      <c r="G55" s="15">
+      <c r="G55" s="14">
         <f t="shared" si="3"/>
         <v>1500</v>
       </c>
-      <c r="H55" s="16" t="s">
-        <v>136</v>
+      <c r="H55" s="15" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
@@ -2402,23 +2373,23 @@
         <v>57</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="E56" s="17">
+        <v>131</v>
+      </c>
+      <c r="E56" s="16">
         <v>0.5</v>
       </c>
-      <c r="F56" s="18">
+      <c r="F56" s="17">
         <v>2000</v>
       </c>
-      <c r="G56" s="18">
+      <c r="G56" s="17">
         <f t="shared" si="3"/>
         <v>1000</v>
       </c>
-      <c r="H56" s="19" t="s">
-        <v>138</v>
+      <c r="H56" s="18" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
@@ -2429,23 +2400,23 @@
         <v>57</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E57" s="14">
+        <v>133</v>
+      </c>
+      <c r="E57" s="19">
         <v>0.5</v>
       </c>
-      <c r="F57" s="15">
+      <c r="F57" s="14">
         <v>3000</v>
       </c>
-      <c r="G57" s="15">
+      <c r="G57" s="14">
         <f t="shared" si="3"/>
         <v>1500</v>
       </c>
-      <c r="H57" s="16" t="s">
-        <v>140</v>
+      <c r="H57" s="15" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
@@ -2453,26 +2424,26 @@
         <v>34</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="E58" s="17">
         <v>100000</v>
       </c>
-      <c r="F58" s="23">
+      <c r="F58" s="16">
         <v>1.2E-2</v>
       </c>
-      <c r="G58" s="18">
+      <c r="G58" s="17">
         <f t="shared" si="3"/>
         <v>1200</v>
       </c>
-      <c r="H58" s="19" t="s">
-        <v>142</v>
+      <c r="H58" s="18" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
@@ -2480,26 +2451,26 @@
         <v>34</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E59" s="14">
         <v>1</v>
       </c>
-      <c r="F59" s="15">
+      <c r="F59" s="14">
         <v>8000</v>
       </c>
-      <c r="G59" s="15">
+      <c r="G59" s="14">
         <f t="shared" si="3"/>
         <v>8000</v>
       </c>
-      <c r="H59" s="16" t="s">
-        <v>144</v>
+      <c r="H59" s="15" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
@@ -2507,26 +2478,26 @@
         <v>34</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E60" s="17">
         <v>100000</v>
       </c>
-      <c r="F60" s="23">
+      <c r="F60" s="16">
         <v>0.06</v>
       </c>
-      <c r="G60" s="18">
+      <c r="G60" s="17">
         <f t="shared" si="3"/>
         <v>6000</v>
       </c>
-      <c r="H60" s="19" t="s">
-        <v>146</v>
+      <c r="H60" s="18" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
@@ -2534,37 +2505,37 @@
         <v>34</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E61" s="14">
+        <v>142</v>
+      </c>
+      <c r="E61" s="19">
         <v>0.5</v>
       </c>
-      <c r="F61" s="15">
+      <c r="F61" s="14">
         <v>2940</v>
       </c>
-      <c r="G61" s="15">
+      <c r="G61" s="14">
         <f t="shared" si="3"/>
         <v>1470</v>
       </c>
-      <c r="H61" s="16" t="s">
-        <v>149</v>
+      <c r="H61" s="15" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A62" s="46" t="s">
-        <v>150</v>
-      </c>
-      <c r="B62" s="35"/>
-      <c r="C62" s="35"/>
-      <c r="D62" s="35"/>
-      <c r="E62" s="35"/>
-      <c r="F62" s="35"/>
+      <c r="A62" s="44" t="s">
+        <v>144</v>
+      </c>
+      <c r="B62" s="33"/>
+      <c r="C62" s="33"/>
+      <c r="D62" s="33"/>
+      <c r="E62" s="33"/>
+      <c r="F62" s="33"/>
       <c r="G62" s="20">
         <f>SUM(G51:G61)</f>
         <v>98670</v>
@@ -2579,23 +2550,23 @@
         <v>57</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E63" s="17">
         <v>1</v>
       </c>
-      <c r="F63" s="18">
+      <c r="F63" s="17">
         <v>15000</v>
       </c>
-      <c r="G63" s="18">
+      <c r="G63" s="17">
         <f t="shared" ref="G63:G74" si="4">E63*F63</f>
         <v>15000</v>
       </c>
-      <c r="H63" s="19" t="s">
-        <v>152</v>
+      <c r="H63" s="18" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
@@ -2606,23 +2577,23 @@
         <v>57</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E64" s="14">
         <v>1</v>
       </c>
-      <c r="F64" s="15">
+      <c r="F64" s="14">
         <v>12000</v>
       </c>
-      <c r="G64" s="15">
+      <c r="G64" s="14">
         <f t="shared" si="4"/>
         <v>12000</v>
       </c>
-      <c r="H64" s="16" t="s">
-        <v>152</v>
+      <c r="H64" s="15" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
@@ -2633,23 +2604,23 @@
         <v>57</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E65" s="17">
         <v>1</v>
       </c>
-      <c r="F65" s="18">
+      <c r="F65" s="17">
         <v>4000</v>
       </c>
-      <c r="G65" s="18">
+      <c r="G65" s="17">
         <f t="shared" si="4"/>
         <v>4000</v>
       </c>
-      <c r="H65" s="19" t="s">
-        <v>152</v>
+      <c r="H65" s="18" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
@@ -2660,23 +2631,23 @@
         <v>57</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E66" s="14">
         <v>1</v>
       </c>
-      <c r="F66" s="15">
+      <c r="F66" s="14">
         <v>3000</v>
       </c>
-      <c r="G66" s="15">
+      <c r="G66" s="14">
         <f t="shared" si="4"/>
         <v>3000</v>
       </c>
-      <c r="H66" s="16" t="s">
-        <v>152</v>
+      <c r="H66" s="15" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
@@ -2687,23 +2658,23 @@
         <v>57</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E67" s="17">
         <v>1</v>
       </c>
-      <c r="F67" s="18">
+      <c r="F67" s="17">
         <v>2000</v>
       </c>
-      <c r="G67" s="18">
+      <c r="G67" s="17">
         <f t="shared" si="4"/>
         <v>2000</v>
       </c>
-      <c r="H67" s="19" t="s">
-        <v>152</v>
+      <c r="H67" s="18" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
@@ -2714,23 +2685,23 @@
         <v>57</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E68" s="14">
         <v>1</v>
       </c>
-      <c r="F68" s="15">
+      <c r="F68" s="14">
         <v>3000</v>
       </c>
-      <c r="G68" s="15">
+      <c r="G68" s="14">
         <f t="shared" si="4"/>
         <v>3000</v>
       </c>
-      <c r="H68" s="16" t="s">
-        <v>152</v>
+      <c r="H68" s="15" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -2738,26 +2709,26 @@
         <v>39</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E69" s="17">
         <v>1</v>
       </c>
-      <c r="F69" s="18">
+      <c r="F69" s="17">
         <v>1200</v>
       </c>
-      <c r="G69" s="18">
+      <c r="G69" s="17">
         <f t="shared" si="4"/>
         <v>1200</v>
       </c>
-      <c r="H69" s="19" t="s">
-        <v>152</v>
+      <c r="H69" s="18" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -2765,26 +2736,26 @@
         <v>39</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="E70" s="14">
         <v>1</v>
       </c>
-      <c r="F70" s="15">
+      <c r="F70" s="14">
         <v>5000</v>
       </c>
-      <c r="G70" s="15">
+      <c r="G70" s="14">
         <f t="shared" si="4"/>
         <v>5000</v>
       </c>
-      <c r="H70" s="16" t="s">
-        <v>154</v>
+      <c r="H70" s="15" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
@@ -2792,26 +2763,26 @@
         <v>39</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E71" s="17">
         <v>1</v>
       </c>
-      <c r="F71" s="18">
+      <c r="F71" s="17">
         <v>6000</v>
       </c>
-      <c r="G71" s="18">
+      <c r="G71" s="17">
         <f t="shared" si="4"/>
         <v>6000</v>
       </c>
-      <c r="H71" s="19" t="s">
-        <v>152</v>
+      <c r="H71" s="18" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
@@ -2819,26 +2790,26 @@
         <v>39</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E72" s="14">
         <v>1</v>
       </c>
-      <c r="F72" s="15">
+      <c r="F72" s="14">
         <v>2940</v>
       </c>
-      <c r="G72" s="15">
+      <c r="G72" s="14">
         <f t="shared" si="4"/>
         <v>2940</v>
       </c>
-      <c r="H72" s="16" t="s">
-        <v>152</v>
+      <c r="H72" s="15" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -2849,23 +2820,23 @@
         <v>57</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E73" s="17">
         <v>1</v>
       </c>
-      <c r="F73" s="18">
+      <c r="F73" s="17">
         <v>1500</v>
       </c>
-      <c r="G73" s="18">
+      <c r="G73" s="17">
         <f t="shared" si="4"/>
         <v>1500</v>
       </c>
-      <c r="H73" s="19" t="s">
-        <v>152</v>
+      <c r="H73" s="18" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
@@ -2876,240 +2847,240 @@
         <v>57</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E74" s="14">
         <v>1</v>
       </c>
-      <c r="F74" s="15">
+      <c r="F74" s="14">
         <v>750</v>
       </c>
-      <c r="G74" s="15">
+      <c r="G74" s="14">
         <f t="shared" si="4"/>
         <v>750</v>
       </c>
-      <c r="H74" s="16" t="s">
-        <v>152</v>
+      <c r="H74" s="15" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A75" s="40" t="s">
-        <v>157</v>
-      </c>
-      <c r="B75" s="38"/>
-      <c r="C75" s="38"/>
-      <c r="D75" s="38"/>
-      <c r="E75" s="38"/>
-      <c r="F75" s="38"/>
-      <c r="G75" s="24">
+      <c r="A75" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="B75" s="36"/>
+      <c r="C75" s="36"/>
+      <c r="D75" s="36"/>
+      <c r="E75" s="36"/>
+      <c r="F75" s="36"/>
+      <c r="G75" s="22">
         <f>SUM(G63:G74)</f>
         <v>56390</v>
       </c>
-      <c r="H75" s="25"/>
+      <c r="H75" s="23"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A78" s="43" t="s">
-        <v>158</v>
-      </c>
-      <c r="B78" s="44"/>
-      <c r="C78" s="44"/>
-      <c r="D78" s="44"/>
-      <c r="E78" s="44"/>
-      <c r="F78" s="44"/>
-      <c r="G78" s="44"/>
-      <c r="H78" s="45"/>
+      <c r="A78" s="41" t="s">
+        <v>152</v>
+      </c>
+      <c r="B78" s="42"/>
+      <c r="C78" s="42"/>
+      <c r="D78" s="42"/>
+      <c r="E78" s="42"/>
+      <c r="F78" s="42"/>
+      <c r="G78" s="42"/>
+      <c r="H78" s="43"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A79" s="49" t="s">
-        <v>159</v>
-      </c>
-      <c r="B79" s="35"/>
-      <c r="C79" s="35"/>
-      <c r="D79" s="35"/>
-      <c r="E79" s="35"/>
-      <c r="F79" s="35"/>
-      <c r="G79" s="35"/>
-      <c r="H79" s="36"/>
+      <c r="A79" s="47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B79" s="33"/>
+      <c r="C79" s="33"/>
+      <c r="D79" s="33"/>
+      <c r="E79" s="33"/>
+      <c r="F79" s="33"/>
+      <c r="G79" s="33"/>
+      <c r="H79" s="34"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="B80" s="50" t="s">
-        <v>161</v>
-      </c>
-      <c r="C80" s="50"/>
-      <c r="D80" s="50"/>
-      <c r="E80" s="50"/>
-      <c r="F80" s="50"/>
-      <c r="G80" s="50"/>
-      <c r="H80" s="51"/>
+        <v>154</v>
+      </c>
+      <c r="B80" s="48" t="s">
+        <v>155</v>
+      </c>
+      <c r="C80" s="48"/>
+      <c r="D80" s="48"/>
+      <c r="E80" s="48"/>
+      <c r="F80" s="48"/>
+      <c r="G80" s="48"/>
+      <c r="H80" s="49"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A81" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="B81" s="53">
+      <c r="A81" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="B81" s="51">
         <f>G30+G38+G50+G62</f>
         <v>322758</v>
       </c>
-      <c r="C81" s="35"/>
-      <c r="D81" s="35"/>
-      <c r="E81" s="35"/>
-      <c r="F81" s="35"/>
-      <c r="G81" s="35"/>
-      <c r="H81" s="36"/>
+      <c r="C81" s="33"/>
+      <c r="D81" s="33"/>
+      <c r="E81" s="33"/>
+      <c r="F81" s="33"/>
+      <c r="G81" s="33"/>
+      <c r="H81" s="34"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A82" s="27" t="s">
-        <v>163</v>
-      </c>
-      <c r="B82" s="59">
+      <c r="A82" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="B82" s="57">
         <f>G75*12</f>
         <v>676680</v>
       </c>
-      <c r="C82" s="32"/>
-      <c r="D82" s="32"/>
-      <c r="E82" s="32"/>
-      <c r="F82" s="32"/>
-      <c r="G82" s="32"/>
-      <c r="H82" s="33"/>
+      <c r="C82" s="30"/>
+      <c r="D82" s="30"/>
+      <c r="E82" s="30"/>
+      <c r="F82" s="30"/>
+      <c r="G82" s="30"/>
+      <c r="H82" s="31"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A83" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="B83" s="34">
+      <c r="A83" s="24" t="s">
+        <v>158</v>
+      </c>
+      <c r="B83" s="32">
         <f>G75/272</f>
         <v>207.31617647058823</v>
       </c>
-      <c r="C83" s="35"/>
-      <c r="D83" s="35"/>
-      <c r="E83" s="35"/>
-      <c r="F83" s="35"/>
-      <c r="G83" s="35"/>
-      <c r="H83" s="36"/>
+      <c r="C83" s="33"/>
+      <c r="D83" s="33"/>
+      <c r="E83" s="33"/>
+      <c r="F83" s="33"/>
+      <c r="G83" s="33"/>
+      <c r="H83" s="34"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A84" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="B84" s="31">
+      <c r="A84" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="B84" s="29">
         <f>G75/100000</f>
         <v>0.56389999999999996</v>
       </c>
-      <c r="C84" s="32"/>
-      <c r="D84" s="32"/>
-      <c r="E84" s="32"/>
-      <c r="F84" s="32"/>
-      <c r="G84" s="32"/>
-      <c r="H84" s="33"/>
+      <c r="C84" s="30"/>
+      <c r="D84" s="30"/>
+      <c r="E84" s="30"/>
+      <c r="F84" s="30"/>
+      <c r="G84" s="30"/>
+      <c r="H84" s="31"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A85" s="26" t="s">
-        <v>166</v>
-      </c>
-      <c r="B85" s="53">
+      <c r="A85" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="B85" s="51">
         <v>200000000</v>
       </c>
-      <c r="C85" s="35"/>
-      <c r="D85" s="35"/>
-      <c r="E85" s="35"/>
-      <c r="F85" s="35"/>
-      <c r="G85" s="35"/>
-      <c r="H85" s="36"/>
+      <c r="C85" s="33"/>
+      <c r="D85" s="33"/>
+      <c r="E85" s="33"/>
+      <c r="F85" s="33"/>
+      <c r="G85" s="33"/>
+      <c r="H85" s="34"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A86" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="B86" s="31">
+      <c r="A86" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="B86" s="29">
         <f>G75*12/200000000</f>
         <v>3.3833999999999999E-3</v>
       </c>
-      <c r="C86" s="32"/>
-      <c r="D86" s="32"/>
-      <c r="E86" s="32"/>
-      <c r="F86" s="32"/>
-      <c r="G86" s="32"/>
-      <c r="H86" s="33"/>
+      <c r="C86" s="30"/>
+      <c r="D86" s="30"/>
+      <c r="E86" s="30"/>
+      <c r="F86" s="30"/>
+      <c r="G86" s="30"/>
+      <c r="H86" s="31"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A87" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="B87" s="53">
+      <c r="A87" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="B87" s="51">
         <v>272</v>
       </c>
-      <c r="C87" s="35"/>
-      <c r="D87" s="35"/>
-      <c r="E87" s="35"/>
-      <c r="F87" s="35"/>
-      <c r="G87" s="35"/>
-      <c r="H87" s="36"/>
+      <c r="C87" s="33"/>
+      <c r="D87" s="33"/>
+      <c r="E87" s="33"/>
+      <c r="F87" s="33"/>
+      <c r="G87" s="33"/>
+      <c r="H87" s="34"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A88" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="B88" s="58" t="s">
+      <c r="A88" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="B88" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="C88" s="32"/>
-      <c r="D88" s="32"/>
-      <c r="E88" s="32"/>
-      <c r="F88" s="32"/>
-      <c r="G88" s="32"/>
-      <c r="H88" s="33"/>
+      <c r="C88" s="30"/>
+      <c r="D88" s="30"/>
+      <c r="E88" s="30"/>
+      <c r="F88" s="30"/>
+      <c r="G88" s="30"/>
+      <c r="H88" s="31"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A89" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="B89" s="53">
+      <c r="A89" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="B89" s="51">
         <v>1200000</v>
       </c>
-      <c r="C89" s="35"/>
-      <c r="D89" s="35"/>
-      <c r="E89" s="35"/>
-      <c r="F89" s="35"/>
-      <c r="G89" s="35"/>
-      <c r="H89" s="36"/>
+      <c r="C89" s="33"/>
+      <c r="D89" s="33"/>
+      <c r="E89" s="33"/>
+      <c r="F89" s="33"/>
+      <c r="G89" s="33"/>
+      <c r="H89" s="34"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A90" s="28"/>
-      <c r="B90" s="29"/>
-      <c r="C90" s="29"/>
-      <c r="D90" s="29"/>
-      <c r="E90" s="29"/>
-      <c r="F90" s="29"/>
-      <c r="G90" s="29"/>
-      <c r="H90" s="30"/>
+      <c r="A90" s="26"/>
+      <c r="B90" s="27"/>
+      <c r="C90" s="27"/>
+      <c r="D90" s="27"/>
+      <c r="E90" s="27"/>
+      <c r="F90" s="27"/>
+      <c r="G90" s="27"/>
+      <c r="H90" s="28"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A91" s="41" t="s">
-        <v>171</v>
-      </c>
-      <c r="B91" s="35"/>
-      <c r="C91" s="35"/>
-      <c r="D91" s="35"/>
-      <c r="E91" s="35"/>
-      <c r="F91" s="35"/>
-      <c r="G91" s="35"/>
-      <c r="H91" s="36"/>
+      <c r="A91" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="B91" s="33"/>
+      <c r="C91" s="33"/>
+      <c r="D91" s="33"/>
+      <c r="E91" s="33"/>
+      <c r="F91" s="33"/>
+      <c r="G91" s="33"/>
+      <c r="H91" s="34"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A92" s="42"/>
-      <c r="B92" s="38"/>
-      <c r="C92" s="38"/>
-      <c r="D92" s="38"/>
-      <c r="E92" s="38"/>
-      <c r="F92" s="38"/>
-      <c r="G92" s="38"/>
-      <c r="H92" s="39"/>
+      <c r="A92" s="40"/>
+      <c r="B92" s="36"/>
+      <c r="C92" s="36"/>
+      <c r="D92" s="36"/>
+      <c r="E92" s="36"/>
+      <c r="F92" s="36"/>
+      <c r="G92" s="36"/>
+      <c r="H92" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="34">

</xml_diff>

<commit_message>
update: Phase 4 complaints to 75K, stipends to Rs. 18,000/month
Phase 4:
- Est. Complaints/Month: 1,00,000 -> 75,000
- Gemini API qty: 100000 -> 75000 (total: 900)
- WhatsApp API qty: 100000 -> 75000 (total: 4,500)
- Phase 4 subtotal: 98,670 -> 79,370 (via SUM formula)

Stipends (all 4 phases):
- Rate: Rs. 25,000 -> Rs. 18,000/person/month
- Unit cost: 12,500 -> 9,000 (half-month)
- Total per phase: 62,500 -> 45,000 (5 x 9,000)

Updated totals (all via formulas):
- Phase 1: 58,250 | Phase 2: 48,750
- Phase 3: 64,588 | Phase 4: 79,370
- Grand Total 1-4: 2,50,958
- Phase 5 monthly: 56,390 (unchanged)
- Annual Maint: 6,76,680 (unchanged)
</commit_message>
<xml_diff>
--- a/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
+++ b/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Delhi-PS-CRM\QuotationSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785ACB68-A2AA-4CD1-8F49-1541300D42EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{531B9D53-498F-452C-AE8C-FB28D3866C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="167">
   <si>
     <t>Delhi PS-CRM — Project Cost Quotation</t>
   </si>
@@ -147,24 +147,27 @@
     <t>Full Delhi Deployment</t>
   </si>
   <si>
-    <t>All 272 wards live, 1,00,000 complaints/month, full system operational</t>
+    <t>All 272 wards live, 75,000 complaints/month, full system operational</t>
+  </si>
+  <si>
+    <t>75,000</t>
+  </si>
+  <si>
+    <t>Phase 5</t>
+  </si>
+  <si>
+    <t>Month 3 onwards</t>
+  </si>
+  <si>
+    <t>Steady State Operations</t>
+  </si>
+  <si>
+    <t>Handed to Delhi government IT team. Maintenance only, quarterly ML retraining</t>
   </si>
   <si>
     <t>1,00,000</t>
   </si>
   <si>
-    <t>Phase 5</t>
-  </si>
-  <si>
-    <t>Month 3 onwards</t>
-  </si>
-  <si>
-    <t>Steady State Operations</t>
-  </si>
-  <si>
-    <t>Handed to Delhi government IT team. Maintenance only, quarterly ML retraining</t>
-  </si>
-  <si>
     <t>Total Project Cost Phases 1-4</t>
   </si>
   <si>
@@ -201,10 +204,10 @@
     <t>Student Developer Stipends</t>
   </si>
   <si>
-    <t>5 students × 2 weeks (0.5 month) @ Rs. 25,000/person/month</t>
-  </si>
-  <si>
-    <t>Rs. 25,000/person/month × 0.5 month × 5 students = Rs. 62,500</t>
+    <t>5 students × 2 weeks (0.5 month) @ Rs. 18,000/person/month</t>
+  </si>
+  <si>
+    <t>Rs. 18,000/person/month × 0.5 month × 5 students = Rs. 45,000</t>
   </si>
   <si>
     <t>Infrastructure</t>
@@ -441,7 +444,7 @@
     <t>WAF enabled</t>
   </si>
   <si>
-    <t>Full-scale classification at 1,00,000 complaints/month</t>
+    <t>Full-scale classification at 75,000 complaints/month</t>
   </si>
   <si>
     <t>Full scale with 30% voice mix</t>
@@ -453,7 +456,7 @@
     <t>Accuracy improves with real data</t>
   </si>
   <si>
-    <t>Full Delhi citizen messaging at 1L conversations/month</t>
+    <t>Full Delhi citizen messaging at 75K conversations/month</t>
   </si>
   <si>
     <t>Peak communication cost</t>
@@ -1386,7 +1389,7 @@
       </c>
       <c r="F14" s="7">
         <f>G30</f>
-        <v>75750</v>
+        <v>58250</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1407,7 +1410,7 @@
       </c>
       <c r="F15" s="11">
         <f>G38</f>
-        <v>66250</v>
+        <v>48750</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -1428,7 +1431,7 @@
       </c>
       <c r="F16" s="7">
         <f>G50</f>
-        <v>82088</v>
+        <v>64588</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -1449,7 +1452,7 @@
       </c>
       <c r="F17" s="11">
         <f>G62</f>
-        <v>98670</v>
+        <v>79370</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1466,7 +1469,7 @@
         <v>42</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F18" s="7">
         <f>G75</f>
@@ -1475,7 +1478,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="50" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B19" s="33"/>
       <c r="C19" s="33"/>
@@ -1483,12 +1486,12 @@
       <c r="E19" s="33"/>
       <c r="F19" s="12">
         <f>G30+G38+G50+G62</f>
-        <v>322758</v>
+        <v>250958</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="55" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" s="36"/>
       <c r="C20" s="36"/>
@@ -1501,7 +1504,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="41" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B22" s="42"/>
       <c r="C22" s="42"/>
@@ -1516,25 +1519,25 @@
         <v>13</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
@@ -1542,26 +1545,26 @@
         <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E24" s="14">
         <v>5</v>
       </c>
       <c r="F24" s="14">
-        <v>12500</v>
+        <v>9000</v>
       </c>
       <c r="G24" s="14">
         <f t="shared" ref="G24:G29" si="0">E24*F24</f>
-        <v>62500</v>
+        <v>45000</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -1569,13 +1572,13 @@
         <v>19</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E25" s="16">
         <v>0.5</v>
@@ -1588,7 +1591,7 @@
         <v>2000</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -1596,13 +1599,13 @@
         <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E26" s="19">
         <v>0.5</v>
@@ -1615,7 +1618,7 @@
         <v>1250</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -1623,13 +1626,13 @@
         <v>19</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E27" s="17">
         <v>1</v>
@@ -1642,7 +1645,7 @@
         <v>5000</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -1650,13 +1653,13 @@
         <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E28" s="14">
         <v>1</v>
@@ -1669,7 +1672,7 @@
         <v>4000</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -1677,13 +1680,13 @@
         <v>19</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E29" s="17">
         <v>1</v>
@@ -1696,12 +1699,12 @@
         <v>1000</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="44" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B30" s="33"/>
       <c r="C30" s="33"/>
@@ -1710,7 +1713,7 @@
       <c r="F30" s="33"/>
       <c r="G30" s="20">
         <f>SUM(G24:G29)</f>
-        <v>75750</v>
+        <v>58250</v>
       </c>
       <c r="H30" s="21"/>
     </row>
@@ -1719,26 +1722,26 @@
         <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E31" s="14">
         <v>5</v>
       </c>
       <c r="F31" s="14">
-        <v>12500</v>
+        <v>9000</v>
       </c>
       <c r="G31" s="14">
         <f t="shared" ref="G31:G37" si="1">E31*F31</f>
-        <v>62500</v>
+        <v>45000</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
@@ -1746,13 +1749,13 @@
         <v>24</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E32" s="16">
         <v>0.5</v>
@@ -1765,7 +1768,7 @@
         <v>2000</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
@@ -1773,13 +1776,13 @@
         <v>24</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E33" s="19">
         <v>0.5</v>
@@ -1792,7 +1795,7 @@
         <v>1250</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
@@ -1800,13 +1803,13 @@
         <v>24</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E34" s="16">
         <v>0.5</v>
@@ -1819,7 +1822,7 @@
         <v>250</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
@@ -1827,13 +1830,13 @@
         <v>24</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E35" s="14">
         <v>1000</v>
@@ -1846,7 +1849,7 @@
         <v>50</v>
       </c>
       <c r="H35" s="15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -1854,13 +1857,13 @@
         <v>24</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E36" s="17">
         <v>1000</v>
@@ -1873,7 +1876,7 @@
         <v>100</v>
       </c>
       <c r="H36" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
@@ -1881,13 +1884,13 @@
         <v>24</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E37" s="14">
         <v>1</v>
@@ -1900,12 +1903,12 @@
         <v>100</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="44" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B38" s="33"/>
       <c r="C38" s="33"/>
@@ -1914,7 +1917,7 @@
       <c r="F38" s="33"/>
       <c r="G38" s="20">
         <f>SUM(G31:G37)</f>
-        <v>66250</v>
+        <v>48750</v>
       </c>
       <c r="H38" s="21"/>
     </row>
@@ -1923,26 +1926,26 @@
         <v>29</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E39" s="17">
         <v>5</v>
       </c>
       <c r="F39" s="17">
-        <v>12500</v>
+        <v>9000</v>
       </c>
       <c r="G39" s="17">
         <f t="shared" ref="G39:G49" si="2">E39*F39</f>
-        <v>62500</v>
+        <v>45000</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
@@ -1950,13 +1953,13 @@
         <v>29</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E40" s="19">
         <v>0.5</v>
@@ -1969,7 +1972,7 @@
         <v>4000</v>
       </c>
       <c r="H40" s="15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
@@ -1977,13 +1980,13 @@
         <v>29</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E41" s="16">
         <v>0.5</v>
@@ -1996,7 +1999,7 @@
         <v>2500</v>
       </c>
       <c r="H41" s="18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
@@ -2004,13 +2007,13 @@
         <v>29</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E42" s="19">
         <v>0.5</v>
@@ -2023,7 +2026,7 @@
         <v>750</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
@@ -2031,13 +2034,13 @@
         <v>29</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E43" s="16">
         <v>0.5</v>
@@ -2050,7 +2053,7 @@
         <v>750</v>
       </c>
       <c r="H43" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
@@ -2058,13 +2061,13 @@
         <v>29</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E44" s="19">
         <v>0.5</v>
@@ -2077,7 +2080,7 @@
         <v>500</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
@@ -2085,13 +2088,13 @@
         <v>29</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E45" s="17">
         <v>20000</v>
@@ -2104,7 +2107,7 @@
         <v>300</v>
       </c>
       <c r="H45" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
@@ -2112,13 +2115,13 @@
         <v>29</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E46" s="14">
         <v>1</v>
@@ -2131,7 +2134,7 @@
         <v>8000</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
@@ -2139,13 +2142,13 @@
         <v>29</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E47" s="17">
         <v>20000</v>
@@ -2158,7 +2161,7 @@
         <v>1200</v>
       </c>
       <c r="H47" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
@@ -2166,13 +2169,13 @@
         <v>29</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E48" s="19">
         <v>0.5</v>
@@ -2185,7 +2188,7 @@
         <v>838</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
@@ -2193,13 +2196,13 @@
         <v>29</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E49" s="16">
         <v>0.5</v>
@@ -2212,12 +2215,12 @@
         <v>750</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="44" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B50" s="33"/>
       <c r="C50" s="33"/>
@@ -2226,7 +2229,7 @@
       <c r="F50" s="33"/>
       <c r="G50" s="20">
         <f>SUM(G39:G49)</f>
-        <v>82088</v>
+        <v>64588</v>
       </c>
       <c r="H50" s="21"/>
     </row>
@@ -2235,26 +2238,26 @@
         <v>34</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E51" s="14">
         <v>5</v>
       </c>
       <c r="F51" s="14">
-        <v>12500</v>
+        <v>9000</v>
       </c>
       <c r="G51" s="14">
         <f t="shared" ref="G51:G61" si="3">E51*F51</f>
-        <v>62500</v>
+        <v>45000</v>
       </c>
       <c r="H51" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
@@ -2262,13 +2265,13 @@
         <v>34</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E52" s="16">
         <v>0.5</v>
@@ -2281,7 +2284,7 @@
         <v>7500</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2289,13 +2292,13 @@
         <v>34</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E53" s="19">
         <v>0.5</v>
@@ -2308,7 +2311,7 @@
         <v>6000</v>
       </c>
       <c r="H53" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
@@ -2316,13 +2319,13 @@
         <v>34</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E54" s="16">
         <v>0.5</v>
@@ -2335,7 +2338,7 @@
         <v>2000</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
@@ -2343,13 +2346,13 @@
         <v>34</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E55" s="19">
         <v>0.5</v>
@@ -2362,7 +2365,7 @@
         <v>1500</v>
       </c>
       <c r="H55" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
@@ -2370,13 +2373,13 @@
         <v>34</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E56" s="16">
         <v>0.5</v>
@@ -2389,7 +2392,7 @@
         <v>1000</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
@@ -2397,13 +2400,13 @@
         <v>34</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E57" s="19">
         <v>0.5</v>
@@ -2416,7 +2419,7 @@
         <v>1500</v>
       </c>
       <c r="H57" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
@@ -2424,26 +2427,26 @@
         <v>34</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E58" s="17">
-        <v>100000</v>
+        <v>75000</v>
       </c>
       <c r="F58" s="16">
         <v>1.2E-2</v>
       </c>
       <c r="G58" s="17">
         <f t="shared" si="3"/>
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
@@ -2451,13 +2454,13 @@
         <v>34</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E59" s="14">
         <v>1</v>
@@ -2470,7 +2473,7 @@
         <v>8000</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
@@ -2478,26 +2481,26 @@
         <v>34</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E60" s="17">
-        <v>100000</v>
+        <v>75000</v>
       </c>
       <c r="F60" s="16">
         <v>0.06</v>
       </c>
       <c r="G60" s="17">
         <f t="shared" si="3"/>
-        <v>6000</v>
+        <v>4500</v>
       </c>
       <c r="H60" s="18" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
@@ -2505,13 +2508,13 @@
         <v>34</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E61" s="19">
         <v>0.5</v>
@@ -2524,12 +2527,12 @@
         <v>1470</v>
       </c>
       <c r="H61" s="15" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="44" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B62" s="33"/>
       <c r="C62" s="33"/>
@@ -2538,7 +2541,7 @@
       <c r="F62" s="33"/>
       <c r="G62" s="20">
         <f>SUM(G51:G61)</f>
-        <v>98670</v>
+        <v>79370</v>
       </c>
       <c r="H62" s="21"/>
     </row>
@@ -2547,13 +2550,13 @@
         <v>39</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E63" s="17">
         <v>1</v>
@@ -2566,7 +2569,7 @@
         <v>15000</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
@@ -2574,13 +2577,13 @@
         <v>39</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E64" s="14">
         <v>1</v>
@@ -2593,7 +2596,7 @@
         <v>12000</v>
       </c>
       <c r="H64" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
@@ -2601,13 +2604,13 @@
         <v>39</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E65" s="17">
         <v>1</v>
@@ -2620,7 +2623,7 @@
         <v>4000</v>
       </c>
       <c r="H65" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
@@ -2628,13 +2631,13 @@
         <v>39</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E66" s="14">
         <v>1</v>
@@ -2647,7 +2650,7 @@
         <v>3000</v>
       </c>
       <c r="H66" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
@@ -2655,13 +2658,13 @@
         <v>39</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E67" s="17">
         <v>1</v>
@@ -2674,7 +2677,7 @@
         <v>2000</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
@@ -2682,13 +2685,13 @@
         <v>39</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E68" s="14">
         <v>1</v>
@@ -2701,7 +2704,7 @@
         <v>3000</v>
       </c>
       <c r="H68" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -2709,13 +2712,13 @@
         <v>39</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E69" s="17">
         <v>1</v>
@@ -2728,7 +2731,7 @@
         <v>1200</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -2736,13 +2739,13 @@
         <v>39</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E70" s="14">
         <v>1</v>
@@ -2755,7 +2758,7 @@
         <v>5000</v>
       </c>
       <c r="H70" s="15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
@@ -2763,13 +2766,13 @@
         <v>39</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E71" s="17">
         <v>1</v>
@@ -2782,7 +2785,7 @@
         <v>6000</v>
       </c>
       <c r="H71" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
@@ -2790,13 +2793,13 @@
         <v>39</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E72" s="14">
         <v>1</v>
@@ -2809,7 +2812,7 @@
         <v>2940</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -2817,13 +2820,13 @@
         <v>39</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E73" s="17">
         <v>1</v>
@@ -2836,7 +2839,7 @@
         <v>1500</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
@@ -2844,13 +2847,13 @@
         <v>39</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E74" s="14">
         <v>1</v>
@@ -2863,12 +2866,12 @@
         <v>750</v>
       </c>
       <c r="H74" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="38" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B75" s="36"/>
       <c r="C75" s="36"/>
@@ -2883,7 +2886,7 @@
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="41" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B78" s="42"/>
       <c r="C78" s="42"/>
@@ -2895,7 +2898,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="47" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B79" s="33"/>
       <c r="C79" s="33"/>
@@ -2907,10 +2910,10 @@
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B80" s="48" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C80" s="48"/>
       <c r="D80" s="48"/>
@@ -2921,11 +2924,11 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B81" s="51">
         <f>G30+G38+G50+G62</f>
-        <v>322758</v>
+        <v>250958</v>
       </c>
       <c r="C81" s="33"/>
       <c r="D81" s="33"/>
@@ -2936,7 +2939,7 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="25" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B82" s="57">
         <f>G75*12</f>
@@ -2951,7 +2954,7 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B83" s="32">
         <f>G75/272</f>
@@ -2966,7 +2969,7 @@
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="25" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B84" s="29">
         <f>G75/100000</f>
@@ -2981,7 +2984,7 @@
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B85" s="51">
         <v>200000000</v>
@@ -2995,7 +2998,7 @@
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="25" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B86" s="29">
         <f>G75*12/200000000</f>
@@ -3010,7 +3013,7 @@
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="24" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B87" s="51">
         <v>272</v>
@@ -3024,7 +3027,7 @@
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="25" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B88" s="56" t="s">
         <v>11</v>
@@ -3038,7 +3041,7 @@
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="24" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B89" s="51">
         <v>1200000</v>
@@ -3062,7 +3065,7 @@
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="39" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B91" s="33"/>
       <c r="C91" s="33"/>

</xml_diff>

<commit_message>
chore: rename team to 5Baddies, add contingency reserves to all phases
</commit_message>
<xml_diff>
--- a/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
+++ b/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Delhi-PS-CRM\QuotationSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{531B9D53-498F-452C-AE8C-FB28D3866C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4354CD33-15F4-43BC-A25B-4BD6D11086FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3768" yWindow="3768" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="171">
   <si>
     <t>Delhi PS-CRM — Project Cost Quotation</t>
   </si>
@@ -42,7 +42,7 @@
     <t>AI-Powered WhatsApp Civic Complaint Management System</t>
   </si>
   <si>
-    <t>Team: Delhi PS-CRM | Document: Cost Quotation v2.0 | Excluding all applicable taxes | All prices in INR</t>
+    <t>Team: 5Baddies | Document: Cost Quotation v2.0 | Excluding all applicable taxes | All prices in INR</t>
   </si>
   <si>
     <t>SECTION 1 — PROJECT OVERVIEW HEADER</t>
@@ -259,6 +259,18 @@
   </si>
   <si>
     <t>Audio API test costs for voice complaints</t>
+  </si>
+  <si>
+    <t>Contingency</t>
+  </si>
+  <si>
+    <t>Contingency Reserve</t>
+  </si>
+  <si>
+    <t>Buffer for unexpected API overages, infra spikes, or integration issues</t>
+  </si>
+  <si>
+    <t>~5% of phase operational costs</t>
   </si>
   <si>
     <t>Phase 1 Subtotal</t>
@@ -857,28 +869,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -887,39 +877,61 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
@@ -1226,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -1238,118 +1250,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="31"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="42" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="33"/>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="50" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="33"/>
       <c r="E6" s="33"/>
       <c r="F6" s="33"/>
       <c r="G6" s="33"/>
-      <c r="H6" s="34"/>
+      <c r="H6" s="39"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="33"/>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="50" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="33"/>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>
       <c r="G7" s="33"/>
-      <c r="H7" s="34"/>
+      <c r="H7" s="39"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="42" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="33"/>
-      <c r="C8" s="52" t="s">
+      <c r="C8" s="50" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="33"/>
       <c r="E8" s="33"/>
       <c r="F8" s="33"/>
       <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="H8" s="39"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="35" t="s">
+      <c r="B9" s="35"/>
+      <c r="C9" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
       <c r="H9" s="37"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="42"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="43"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="31"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -1388,8 +1400,8 @@
         <v>23</v>
       </c>
       <c r="F14" s="7">
-        <f>G30</f>
-        <v>58250</v>
+        <f>G31</f>
+        <v>60750</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1409,8 +1421,8 @@
         <v>28</v>
       </c>
       <c r="F15" s="11">
-        <f>G38</f>
-        <v>48750</v>
+        <f>G40</f>
+        <v>51250</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -1430,8 +1442,8 @@
         <v>33</v>
       </c>
       <c r="F16" s="7">
-        <f>G50</f>
-        <v>64588</v>
+        <f>G53</f>
+        <v>68588</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -1451,8 +1463,8 @@
         <v>38</v>
       </c>
       <c r="F17" s="11">
-        <f>G62</f>
-        <v>79370</v>
+        <f>G66</f>
+        <v>83370</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1472,12 +1484,12 @@
         <v>43</v>
       </c>
       <c r="F18" s="7">
-        <f>G75</f>
-        <v>56390</v>
+        <f>G80</f>
+        <v>58890</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="42" t="s">
         <v>44</v>
       </c>
       <c r="B19" s="33"/>
@@ -1485,34 +1497,34 @@
       <c r="D19" s="33"/>
       <c r="E19" s="33"/>
       <c r="F19" s="12">
-        <f>G30+G38+G50+G62</f>
-        <v>250958</v>
+        <f>G31+G40+G53+G66</f>
+        <v>263958</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
       <c r="F20" s="13">
-        <f>G75*12</f>
-        <v>676680</v>
+        <f>G80*12</f>
+        <v>706680</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="41" t="s">
+      <c r="A22" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="43"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="31"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
@@ -1560,7 +1572,7 @@
         <v>9000</v>
       </c>
       <c r="G24" s="14">
-        <f t="shared" ref="G24:G29" si="0">E24*F24</f>
+        <f t="shared" ref="G24:G30" si="0">E24*F24</f>
         <v>45000</v>
       </c>
       <c r="H24" s="15" t="s">
@@ -1703,72 +1715,72 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="44" t="s">
+      <c r="A30" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B30" s="33"/>
-      <c r="C30" s="33"/>
-      <c r="D30" s="33"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="20">
-        <f>SUM(G24:G29)</f>
-        <v>58250</v>
-      </c>
-      <c r="H30" s="21"/>
+      <c r="C30" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30" s="14">
+        <v>1</v>
+      </c>
+      <c r="F30" s="14">
+        <v>2500</v>
+      </c>
+      <c r="G30" s="14">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E31" s="14">
-        <v>5</v>
-      </c>
-      <c r="F31" s="14">
-        <v>9000</v>
-      </c>
-      <c r="G31" s="14">
-        <f t="shared" ref="G31:G37" si="1">E31*F31</f>
-        <v>45000</v>
-      </c>
-      <c r="H31" s="15" t="s">
-        <v>57</v>
-      </c>
+      <c r="A31" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" s="33"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="20">
+        <f>SUM(G24:G30)</f>
+        <v>60750</v>
+      </c>
+      <c r="H31" s="21"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>24</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E32" s="16">
-        <v>0.5</v>
+        <v>56</v>
+      </c>
+      <c r="E32" s="17">
+        <v>5</v>
       </c>
       <c r="F32" s="17">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="G32" s="17">
-        <f t="shared" si="1"/>
-        <v>2000</v>
+        <f t="shared" ref="G32:G39" si="1">E32*F32</f>
+        <v>45000</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
@@ -1779,23 +1791,23 @@
         <v>58</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E33" s="19">
         <v>0.5</v>
       </c>
       <c r="F33" s="14">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="G33" s="14">
         <f t="shared" si="1"/>
-        <v>1250</v>
+        <v>2000</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
@@ -1806,23 +1818,23 @@
         <v>58</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E34" s="16">
         <v>0.5</v>
       </c>
       <c r="F34" s="17">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="G34" s="17">
         <f t="shared" si="1"/>
-        <v>250</v>
+        <v>1250</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
@@ -1830,7 +1842,7 @@
         <v>24</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>86</v>
@@ -1838,21 +1850,21 @@
       <c r="D35" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E35" s="14">
-        <v>1000</v>
-      </c>
-      <c r="F35" s="19">
-        <v>0.05</v>
+      <c r="E35" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="F35" s="14">
+        <v>500</v>
       </c>
       <c r="G35" s="14">
         <f t="shared" si="1"/>
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="H35" s="15" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
         <v>24</v>
       </c>
@@ -1869,137 +1881,137 @@
         <v>1000</v>
       </c>
       <c r="F36" s="16">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G36" s="17">
         <f t="shared" si="1"/>
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H36" s="18" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E37" s="14">
-        <v>1</v>
-      </c>
-      <c r="F37" s="14">
-        <v>100</v>
+        <v>1000</v>
+      </c>
+      <c r="F37" s="19">
+        <v>0.1</v>
       </c>
       <c r="G37" s="14">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="44" t="s">
-        <v>96</v>
-      </c>
-      <c r="B38" s="33"/>
-      <c r="C38" s="33"/>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="20">
-        <f>SUM(G31:G37)</f>
-        <v>48750</v>
-      </c>
-      <c r="H38" s="21"/>
+      <c r="A38" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E38" s="17">
+        <v>1</v>
+      </c>
+      <c r="F38" s="17">
+        <v>100</v>
+      </c>
+      <c r="G38" s="17">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="H38" s="18" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="E39" s="17">
-        <v>5</v>
-      </c>
-      <c r="F39" s="17">
-        <v>9000</v>
-      </c>
-      <c r="G39" s="17">
-        <f t="shared" ref="G39:G49" si="2">E39*F39</f>
-        <v>45000</v>
-      </c>
-      <c r="H39" s="18" t="s">
-        <v>57</v>
+      <c r="A39" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E39" s="14">
+        <v>1</v>
+      </c>
+      <c r="F39" s="14">
+        <v>2500</v>
+      </c>
+      <c r="G39" s="14">
+        <f t="shared" si="1"/>
+        <v>2500</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E40" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="F40" s="14">
-        <v>8000</v>
-      </c>
-      <c r="G40" s="14">
-        <f t="shared" si="2"/>
-        <v>4000</v>
-      </c>
-      <c r="H40" s="15" t="s">
-        <v>98</v>
-      </c>
+      <c r="A40" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B40" s="33"/>
+      <c r="C40" s="33"/>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="20">
+        <f>SUM(G32:G39)</f>
+        <v>51250</v>
+      </c>
+      <c r="H40" s="21"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>29</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E41" s="16">
-        <v>0.5</v>
+        <v>56</v>
+      </c>
+      <c r="E41" s="17">
+        <v>5</v>
       </c>
       <c r="F41" s="17">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="G41" s="17">
-        <f t="shared" si="2"/>
-        <v>2500</v>
+        <f t="shared" ref="G41:G52" si="2">E41*F41</f>
+        <v>45000</v>
       </c>
       <c r="H41" s="18" t="s">
-        <v>101</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.3">
@@ -2010,23 +2022,23 @@
         <v>58</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E42" s="19">
         <v>0.5</v>
       </c>
       <c r="F42" s="14">
-        <v>1500</v>
+        <v>8000</v>
       </c>
       <c r="G42" s="14">
         <f t="shared" si="2"/>
-        <v>750</v>
+        <v>4000</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
@@ -2037,23 +2049,23 @@
         <v>58</v>
       </c>
       <c r="C43" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>105</v>
       </c>
       <c r="E43" s="16">
         <v>0.5</v>
       </c>
       <c r="F43" s="17">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="G43" s="17">
         <f t="shared" si="2"/>
-        <v>750</v>
+        <v>2500</v>
       </c>
       <c r="H43" s="18" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
@@ -2064,23 +2076,23 @@
         <v>58</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E44" s="19">
         <v>0.5</v>
       </c>
       <c r="F44" s="14">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="G44" s="14">
         <f t="shared" si="2"/>
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
@@ -2088,26 +2100,26 @@
         <v>29</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="E45" s="17">
-        <v>20000</v>
-      </c>
-      <c r="F45" s="16">
-        <v>1.4999999999999999E-2</v>
+        <v>109</v>
+      </c>
+      <c r="E45" s="16">
+        <v>0.5</v>
+      </c>
+      <c r="F45" s="17">
+        <v>1500</v>
       </c>
       <c r="G45" s="17">
         <f t="shared" si="2"/>
-        <v>300</v>
+        <v>750</v>
       </c>
       <c r="H45" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
@@ -2115,26 +2127,26 @@
         <v>29</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="E46" s="14">
-        <v>1</v>
+      <c r="E46" s="19">
+        <v>0.5</v>
       </c>
       <c r="F46" s="14">
-        <v>8000</v>
+        <v>1000</v>
       </c>
       <c r="G46" s="14">
         <f t="shared" si="2"/>
-        <v>8000</v>
+        <v>500</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
@@ -2148,20 +2160,20 @@
         <v>90</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E47" s="17">
         <v>20000</v>
       </c>
       <c r="F47" s="16">
-        <v>0.06</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="G47" s="17">
         <f t="shared" si="2"/>
-        <v>1200</v>
+        <v>300</v>
       </c>
       <c r="H47" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
@@ -2172,23 +2184,23 @@
         <v>89</v>
       </c>
       <c r="C48" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D48" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E48" s="19">
-        <v>0.5</v>
+      <c r="E48" s="14">
+        <v>1</v>
       </c>
       <c r="F48" s="14">
-        <v>1676</v>
+        <v>8000</v>
       </c>
       <c r="G48" s="14">
         <f t="shared" si="2"/>
-        <v>838</v>
+        <v>8000</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
@@ -2196,149 +2208,149 @@
         <v>29</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>120</v>
+        <v>94</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E49" s="16">
-        <v>0.5</v>
-      </c>
-      <c r="F49" s="17">
-        <v>1500</v>
+        <v>119</v>
+      </c>
+      <c r="E49" s="17">
+        <v>20000</v>
+      </c>
+      <c r="F49" s="16">
+        <v>0.06</v>
       </c>
       <c r="G49" s="17">
         <f t="shared" si="2"/>
+        <v>1200</v>
+      </c>
+      <c r="H49" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E50" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="F50" s="14">
+        <v>1676</v>
+      </c>
+      <c r="G50" s="14">
+        <f t="shared" si="2"/>
+        <v>838</v>
+      </c>
+      <c r="H50" s="15" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="E51" s="16">
+        <v>0.5</v>
+      </c>
+      <c r="F51" s="17">
+        <v>1500</v>
+      </c>
+      <c r="G51" s="17">
+        <f t="shared" si="2"/>
         <v>750</v>
       </c>
-      <c r="H49" s="18" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="44" t="s">
-        <v>123</v>
-      </c>
-      <c r="B50" s="33"/>
-      <c r="C50" s="33"/>
-      <c r="D50" s="33"/>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="20">
-        <f>SUM(G39:G49)</f>
-        <v>64588</v>
-      </c>
-      <c r="H50" s="21"/>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E51" s="14">
-        <v>5</v>
-      </c>
-      <c r="F51" s="14">
-        <v>9000</v>
-      </c>
-      <c r="G51" s="14">
-        <f t="shared" ref="G51:G61" si="3">E51*F51</f>
-        <v>45000</v>
-      </c>
-      <c r="H51" s="15" t="s">
-        <v>57</v>
+      <c r="H51" s="18" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C52" s="9" t="s">
+      <c r="A52" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="E52" s="16">
-        <v>0.5</v>
-      </c>
-      <c r="F52" s="17">
-        <v>15000</v>
-      </c>
-      <c r="G52" s="17">
-        <f t="shared" si="3"/>
-        <v>7500</v>
-      </c>
-      <c r="H52" s="18" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E53" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="F53" s="14">
-        <v>12000</v>
-      </c>
-      <c r="G53" s="14">
-        <f t="shared" si="3"/>
-        <v>6000</v>
-      </c>
-      <c r="H53" s="15" t="s">
+      <c r="D52" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E52" s="14">
+        <v>1</v>
+      </c>
+      <c r="F52" s="14">
+        <v>4000</v>
+      </c>
+      <c r="G52" s="14">
+        <f t="shared" si="2"/>
+        <v>4000</v>
+      </c>
+      <c r="H52" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" s="32" t="s">
         <v>127</v>
       </c>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="33"/>
+      <c r="E53" s="33"/>
+      <c r="F53" s="33"/>
+      <c r="G53" s="20">
+        <f>SUM(G41:G52)</f>
+        <v>68588</v>
+      </c>
+      <c r="H53" s="21"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="E54" s="16">
-        <v>0.5</v>
+        <v>56</v>
+      </c>
+      <c r="E54" s="17">
+        <v>5</v>
       </c>
       <c r="F54" s="17">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="G54" s="17">
-        <f t="shared" si="3"/>
-        <v>2000</v>
+        <f t="shared" ref="G54:G65" si="3">E54*F54</f>
+        <v>45000</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>129</v>
+        <v>57</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
@@ -2349,26 +2361,26 @@
         <v>58</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E55" s="19">
         <v>0.5</v>
       </c>
       <c r="F55" s="14">
-        <v>3000</v>
+        <v>15000</v>
       </c>
       <c r="G55" s="14">
         <f t="shared" si="3"/>
-        <v>1500</v>
+        <v>7500</v>
       </c>
       <c r="H55" s="15" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
         <v>34</v>
       </c>
@@ -2376,23 +2388,23 @@
         <v>58</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E56" s="16">
         <v>0.5</v>
       </c>
       <c r="F56" s="17">
-        <v>2000</v>
+        <v>12000</v>
       </c>
       <c r="G56" s="17">
         <f t="shared" si="3"/>
-        <v>1000</v>
+        <v>6000</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
@@ -2403,23 +2415,23 @@
         <v>58</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>120</v>
+        <v>86</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E57" s="19">
         <v>0.5</v>
       </c>
       <c r="F57" s="14">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="G57" s="14">
         <f t="shared" si="3"/>
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="H57" s="15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
@@ -2427,26 +2439,26 @@
         <v>34</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="E58" s="17">
-        <v>75000</v>
-      </c>
-      <c r="F58" s="16">
-        <v>1.2E-2</v>
+        <v>134</v>
+      </c>
+      <c r="E58" s="16">
+        <v>0.5</v>
+      </c>
+      <c r="F58" s="17">
+        <v>3000</v>
       </c>
       <c r="G58" s="17">
         <f t="shared" si="3"/>
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
@@ -2454,26 +2466,26 @@
         <v>34</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="E59" s="14">
-        <v>1</v>
+        <v>136</v>
+      </c>
+      <c r="E59" s="19">
+        <v>0.5</v>
       </c>
       <c r="F59" s="14">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="G59" s="14">
         <f t="shared" si="3"/>
-        <v>8000</v>
+        <v>1000</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
@@ -2481,26 +2493,26 @@
         <v>34</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="E60" s="17">
-        <v>75000</v>
-      </c>
-      <c r="F60" s="16">
-        <v>0.06</v>
+        <v>138</v>
+      </c>
+      <c r="E60" s="16">
+        <v>0.5</v>
+      </c>
+      <c r="F60" s="17">
+        <v>3000</v>
       </c>
       <c r="G60" s="17">
         <f t="shared" si="3"/>
-        <v>4500</v>
+        <v>1500</v>
       </c>
       <c r="H60" s="18" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
@@ -2511,147 +2523,147 @@
         <v>89</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>142</v>
+        <v>90</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="E61" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="F61" s="14">
-        <v>2940</v>
+        <v>140</v>
+      </c>
+      <c r="E61" s="14">
+        <v>75000</v>
+      </c>
+      <c r="F61" s="19">
+        <v>1.2E-2</v>
       </c>
       <c r="G61" s="14">
         <f t="shared" si="3"/>
+        <v>900</v>
+      </c>
+      <c r="H61" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A62" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="E62" s="17">
+        <v>1</v>
+      </c>
+      <c r="F62" s="17">
+        <v>8000</v>
+      </c>
+      <c r="G62" s="17">
+        <f t="shared" si="3"/>
+        <v>8000</v>
+      </c>
+      <c r="H62" s="18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E63" s="14">
+        <v>75000</v>
+      </c>
+      <c r="F63" s="19">
+        <v>0.06</v>
+      </c>
+      <c r="G63" s="14">
+        <f t="shared" si="3"/>
+        <v>4500</v>
+      </c>
+      <c r="H63" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A64" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E64" s="16">
+        <v>0.5</v>
+      </c>
+      <c r="F64" s="17">
+        <v>2940</v>
+      </c>
+      <c r="G64" s="17">
+        <f t="shared" si="3"/>
         <v>1470</v>
       </c>
-      <c r="H61" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A62" s="44" t="s">
-        <v>145</v>
-      </c>
-      <c r="B62" s="33"/>
-      <c r="C62" s="33"/>
-      <c r="D62" s="33"/>
-      <c r="E62" s="33"/>
-      <c r="F62" s="33"/>
-      <c r="G62" s="20">
-        <f>SUM(G51:G61)</f>
-        <v>79370</v>
-      </c>
-      <c r="H62" s="21"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A63" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B63" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C63" s="9" t="s">
+      <c r="H64" s="18" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D63" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="E63" s="17">
+      <c r="D65" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E65" s="14">
         <v>1</v>
       </c>
-      <c r="F63" s="17">
-        <v>15000</v>
-      </c>
-      <c r="G63" s="17">
-        <f t="shared" ref="G63:G74" si="4">E63*F63</f>
-        <v>15000</v>
-      </c>
-      <c r="H63" s="18" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="E64" s="14">
-        <v>1</v>
-      </c>
-      <c r="F64" s="14">
-        <v>12000</v>
-      </c>
-      <c r="G64" s="14">
-        <f t="shared" si="4"/>
-        <v>12000</v>
-      </c>
-      <c r="H64" s="15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A65" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B65" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C65" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="E65" s="17">
-        <v>1</v>
-      </c>
-      <c r="F65" s="17">
+      <c r="F65" s="14">
         <v>4000</v>
       </c>
-      <c r="G65" s="17">
-        <f t="shared" si="4"/>
+      <c r="G65" s="14">
+        <f t="shared" si="3"/>
         <v>4000</v>
       </c>
-      <c r="H65" s="18" t="s">
-        <v>147</v>
+      <c r="H65" s="15" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="E66" s="14">
-        <v>1</v>
-      </c>
-      <c r="F66" s="14">
-        <v>3000</v>
-      </c>
-      <c r="G66" s="14">
-        <f t="shared" si="4"/>
-        <v>3000</v>
-      </c>
-      <c r="H66" s="15" t="s">
-        <v>147</v>
-      </c>
+      <c r="A66" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="B66" s="33"/>
+      <c r="C66" s="33"/>
+      <c r="D66" s="33"/>
+      <c r="E66" s="33"/>
+      <c r="F66" s="33"/>
+      <c r="G66" s="20">
+        <f>SUM(G54:G65)</f>
+        <v>83370</v>
+      </c>
+      <c r="H66" s="21"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="8" t="s">
@@ -2661,23 +2673,23 @@
         <v>58</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E67" s="17">
         <v>1</v>
       </c>
       <c r="F67" s="17">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="G67" s="17">
-        <f t="shared" si="4"/>
-        <v>2000</v>
+        <f t="shared" ref="G67:G79" si="4">E67*F67</f>
+        <v>15000</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
@@ -2688,23 +2700,23 @@
         <v>58</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>120</v>
+        <v>83</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E68" s="14">
         <v>1</v>
       </c>
       <c r="F68" s="14">
-        <v>3000</v>
+        <v>12000</v>
       </c>
       <c r="G68" s="14">
         <f t="shared" si="4"/>
-        <v>3000</v>
+        <v>12000</v>
       </c>
       <c r="H68" s="15" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -2712,26 +2724,26 @@
         <v>39</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C69" s="9" t="s">
         <v>86</v>
       </c>
       <c r="D69" s="9" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E69" s="17">
         <v>1</v>
       </c>
       <c r="F69" s="17">
-        <v>1200</v>
+        <v>4000</v>
       </c>
       <c r="G69" s="17">
         <f t="shared" si="4"/>
-        <v>1200</v>
+        <v>4000</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -2739,26 +2751,26 @@
         <v>39</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E70" s="14">
         <v>1</v>
       </c>
       <c r="F70" s="14">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="G70" s="14">
         <f t="shared" si="4"/>
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="H70" s="15" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
@@ -2766,26 +2778,26 @@
         <v>39</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E71" s="17">
         <v>1</v>
       </c>
       <c r="F71" s="17">
-        <v>6000</v>
+        <v>2000</v>
       </c>
       <c r="G71" s="17">
         <f t="shared" si="4"/>
-        <v>6000</v>
+        <v>2000</v>
       </c>
       <c r="H71" s="18" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
@@ -2793,26 +2805,26 @@
         <v>39</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E72" s="14">
         <v>1</v>
       </c>
       <c r="F72" s="14">
-        <v>2940</v>
+        <v>3000</v>
       </c>
       <c r="G72" s="14">
         <f t="shared" si="4"/>
-        <v>2940</v>
+        <v>3000</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -2820,26 +2832,26 @@
         <v>39</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C73" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D73" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="D73" s="9" t="s">
-        <v>146</v>
       </c>
       <c r="E73" s="17">
         <v>1</v>
       </c>
       <c r="F73" s="17">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="G73" s="17">
         <f t="shared" si="4"/>
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
@@ -2847,280 +2859,415 @@
         <v>39</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>151</v>
+        <v>116</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="E74" s="14">
         <v>1</v>
       </c>
       <c r="F74" s="14">
-        <v>750</v>
+        <v>5000</v>
       </c>
       <c r="G74" s="14">
         <f t="shared" si="4"/>
+        <v>5000</v>
+      </c>
+      <c r="H74" s="15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A75" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E75" s="17">
+        <v>1</v>
+      </c>
+      <c r="F75" s="17">
+        <v>6000</v>
+      </c>
+      <c r="G75" s="17">
+        <f t="shared" si="4"/>
+        <v>6000</v>
+      </c>
+      <c r="H75" s="18" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E76" s="14">
+        <v>1</v>
+      </c>
+      <c r="F76" s="14">
+        <v>2940</v>
+      </c>
+      <c r="G76" s="14">
+        <f t="shared" si="4"/>
+        <v>2940</v>
+      </c>
+      <c r="H76" s="15" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E77" s="17">
+        <v>1</v>
+      </c>
+      <c r="F77" s="17">
+        <v>1500</v>
+      </c>
+      <c r="G77" s="17">
+        <f t="shared" si="4"/>
+        <v>1500</v>
+      </c>
+      <c r="H77" s="18" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E78" s="14">
+        <v>1</v>
+      </c>
+      <c r="F78" s="14">
         <v>750</v>
       </c>
-      <c r="H74" s="15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A75" s="38" t="s">
-        <v>152</v>
-      </c>
-      <c r="B75" s="36"/>
-      <c r="C75" s="36"/>
-      <c r="D75" s="36"/>
-      <c r="E75" s="36"/>
-      <c r="F75" s="36"/>
-      <c r="G75" s="22">
-        <f>SUM(G63:G74)</f>
-        <v>56390</v>
-      </c>
-      <c r="H75" s="23"/>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A78" s="41" t="s">
-        <v>153</v>
-      </c>
-      <c r="B78" s="42"/>
-      <c r="C78" s="42"/>
-      <c r="D78" s="42"/>
-      <c r="E78" s="42"/>
-      <c r="F78" s="42"/>
-      <c r="G78" s="42"/>
-      <c r="H78" s="43"/>
+      <c r="G78" s="14">
+        <f t="shared" si="4"/>
+        <v>750</v>
+      </c>
+      <c r="H78" s="15" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A79" s="47" t="s">
-        <v>154</v>
-      </c>
-      <c r="B79" s="33"/>
-      <c r="C79" s="33"/>
-      <c r="D79" s="33"/>
-      <c r="E79" s="33"/>
-      <c r="F79" s="33"/>
-      <c r="G79" s="33"/>
-      <c r="H79" s="34"/>
+      <c r="A79" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E79" s="17">
+        <v>1</v>
+      </c>
+      <c r="F79" s="17">
+        <v>2500</v>
+      </c>
+      <c r="G79" s="17">
+        <f t="shared" si="4"/>
+        <v>2500</v>
+      </c>
+      <c r="H79" s="18" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A80" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B80" s="48" t="s">
+      <c r="A80" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="C80" s="48"/>
-      <c r="D80" s="48"/>
-      <c r="E80" s="48"/>
-      <c r="F80" s="48"/>
-      <c r="G80" s="48"/>
-      <c r="H80" s="49"/>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A81" s="24" t="s">
+      <c r="B80" s="35"/>
+      <c r="C80" s="35"/>
+      <c r="D80" s="35"/>
+      <c r="E80" s="35"/>
+      <c r="F80" s="35"/>
+      <c r="G80" s="22">
+        <f>SUM(G67:G79)</f>
+        <v>58890</v>
+      </c>
+      <c r="H80" s="23"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A83" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="B81" s="51">
-        <f>G30+G38+G50+G62</f>
-        <v>250958</v>
-      </c>
-      <c r="C81" s="33"/>
-      <c r="D81" s="33"/>
-      <c r="E81" s="33"/>
-      <c r="F81" s="33"/>
-      <c r="G81" s="33"/>
-      <c r="H81" s="34"/>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A82" s="25" t="s">
+      <c r="B83" s="30"/>
+      <c r="C83" s="30"/>
+      <c r="D83" s="30"/>
+      <c r="E83" s="30"/>
+      <c r="F83" s="30"/>
+      <c r="G83" s="30"/>
+      <c r="H83" s="31"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A84" s="51" t="s">
         <v>158</v>
       </c>
-      <c r="B82" s="57">
-        <f>G75*12</f>
-        <v>676680</v>
-      </c>
-      <c r="C82" s="30"/>
-      <c r="D82" s="30"/>
-      <c r="E82" s="30"/>
-      <c r="F82" s="30"/>
-      <c r="G82" s="30"/>
-      <c r="H82" s="31"/>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A83" s="24" t="s">
+      <c r="B84" s="33"/>
+      <c r="C84" s="33"/>
+      <c r="D84" s="33"/>
+      <c r="E84" s="33"/>
+      <c r="F84" s="33"/>
+      <c r="G84" s="33"/>
+      <c r="H84" s="39"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A85" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B83" s="32">
-        <f>G75/272</f>
-        <v>207.31617647058823</v>
-      </c>
-      <c r="C83" s="33"/>
-      <c r="D83" s="33"/>
-      <c r="E83" s="33"/>
-      <c r="F83" s="33"/>
-      <c r="G83" s="33"/>
-      <c r="H83" s="34"/>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A84" s="25" t="s">
+      <c r="B85" s="46" t="s">
         <v>160</v>
       </c>
-      <c r="B84" s="29">
-        <f>G75/100000</f>
-        <v>0.56389999999999996</v>
-      </c>
-      <c r="C84" s="30"/>
-      <c r="D84" s="30"/>
-      <c r="E84" s="30"/>
-      <c r="F84" s="30"/>
-      <c r="G84" s="30"/>
-      <c r="H84" s="31"/>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A85" s="24" t="s">
+      <c r="C85" s="46"/>
+      <c r="D85" s="46"/>
+      <c r="E85" s="46"/>
+      <c r="F85" s="46"/>
+      <c r="G85" s="46"/>
+      <c r="H85" s="47"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A86" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="B85" s="51">
+      <c r="B86" s="38">
+        <f>G31+G40+G53+G66</f>
+        <v>263958</v>
+      </c>
+      <c r="C86" s="33"/>
+      <c r="D86" s="33"/>
+      <c r="E86" s="33"/>
+      <c r="F86" s="33"/>
+      <c r="G86" s="33"/>
+      <c r="H86" s="39"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A87" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="B87" s="57">
+        <f>G80*12</f>
+        <v>706680</v>
+      </c>
+      <c r="C87" s="44"/>
+      <c r="D87" s="44"/>
+      <c r="E87" s="44"/>
+      <c r="F87" s="44"/>
+      <c r="G87" s="44"/>
+      <c r="H87" s="45"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A88" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="B88" s="56">
+        <f>G80/272</f>
+        <v>216.50735294117646</v>
+      </c>
+      <c r="C88" s="33"/>
+      <c r="D88" s="33"/>
+      <c r="E88" s="33"/>
+      <c r="F88" s="33"/>
+      <c r="G88" s="33"/>
+      <c r="H88" s="39"/>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A89" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="B89" s="43">
+        <f>G80/100000</f>
+        <v>0.58889999999999998</v>
+      </c>
+      <c r="C89" s="44"/>
+      <c r="D89" s="44"/>
+      <c r="E89" s="44"/>
+      <c r="F89" s="44"/>
+      <c r="G89" s="44"/>
+      <c r="H89" s="45"/>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A90" s="24" t="s">
+        <v>165</v>
+      </c>
+      <c r="B90" s="38">
         <v>200000000</v>
       </c>
-      <c r="C85" s="33"/>
-      <c r="D85" s="33"/>
-      <c r="E85" s="33"/>
-      <c r="F85" s="33"/>
-      <c r="G85" s="33"/>
-      <c r="H85" s="34"/>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A86" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="B86" s="29">
-        <f>G75*12/200000000</f>
-        <v>3.3833999999999999E-3</v>
-      </c>
-      <c r="C86" s="30"/>
-      <c r="D86" s="30"/>
-      <c r="E86" s="30"/>
-      <c r="F86" s="30"/>
-      <c r="G86" s="30"/>
-      <c r="H86" s="31"/>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A87" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="B87" s="51">
+      <c r="C90" s="33"/>
+      <c r="D90" s="33"/>
+      <c r="E90" s="33"/>
+      <c r="F90" s="33"/>
+      <c r="G90" s="33"/>
+      <c r="H90" s="39"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A91" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="B91" s="43">
+        <f>G80*12/200000000</f>
+        <v>3.5333999999999999E-3</v>
+      </c>
+      <c r="C91" s="44"/>
+      <c r="D91" s="44"/>
+      <c r="E91" s="44"/>
+      <c r="F91" s="44"/>
+      <c r="G91" s="44"/>
+      <c r="H91" s="45"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A92" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="B92" s="38">
         <v>272</v>
       </c>
-      <c r="C87" s="33"/>
-      <c r="D87" s="33"/>
-      <c r="E87" s="33"/>
-      <c r="F87" s="33"/>
-      <c r="G87" s="33"/>
-      <c r="H87" s="34"/>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A88" s="25" t="s">
-        <v>164</v>
-      </c>
-      <c r="B88" s="56" t="s">
+      <c r="C92" s="33"/>
+      <c r="D92" s="33"/>
+      <c r="E92" s="33"/>
+      <c r="F92" s="33"/>
+      <c r="G92" s="33"/>
+      <c r="H92" s="39"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A93" s="25" t="s">
+        <v>168</v>
+      </c>
+      <c r="B93" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="C88" s="30"/>
-      <c r="D88" s="30"/>
-      <c r="E88" s="30"/>
-      <c r="F88" s="30"/>
-      <c r="G88" s="30"/>
-      <c r="H88" s="31"/>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A89" s="24" t="s">
-        <v>165</v>
-      </c>
-      <c r="B89" s="51">
+      <c r="C93" s="44"/>
+      <c r="D93" s="44"/>
+      <c r="E93" s="44"/>
+      <c r="F93" s="44"/>
+      <c r="G93" s="44"/>
+      <c r="H93" s="45"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A94" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="B94" s="38">
         <v>1200000</v>
       </c>
-      <c r="C89" s="33"/>
-      <c r="D89" s="33"/>
-      <c r="E89" s="33"/>
-      <c r="F89" s="33"/>
-      <c r="G89" s="33"/>
-      <c r="H89" s="34"/>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A90" s="26"/>
-      <c r="B90" s="27"/>
-      <c r="C90" s="27"/>
-      <c r="D90" s="27"/>
-      <c r="E90" s="27"/>
-      <c r="F90" s="27"/>
-      <c r="G90" s="27"/>
-      <c r="H90" s="28"/>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A91" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="B91" s="33"/>
-      <c r="C91" s="33"/>
-      <c r="D91" s="33"/>
-      <c r="E91" s="33"/>
-      <c r="F91" s="33"/>
-      <c r="G91" s="33"/>
-      <c r="H91" s="34"/>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A92" s="40"/>
-      <c r="B92" s="36"/>
-      <c r="C92" s="36"/>
-      <c r="D92" s="36"/>
-      <c r="E92" s="36"/>
-      <c r="F92" s="36"/>
-      <c r="G92" s="36"/>
-      <c r="H92" s="37"/>
+      <c r="C94" s="33"/>
+      <c r="D94" s="33"/>
+      <c r="E94" s="33"/>
+      <c r="F94" s="33"/>
+      <c r="G94" s="33"/>
+      <c r="H94" s="39"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A95" s="26"/>
+      <c r="B95" s="27"/>
+      <c r="C95" s="27"/>
+      <c r="D95" s="27"/>
+      <c r="E95" s="27"/>
+      <c r="F95" s="27"/>
+      <c r="G95" s="27"/>
+      <c r="H95" s="28"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A96" s="48" t="s">
+        <v>170</v>
+      </c>
+      <c r="B96" s="33"/>
+      <c r="C96" s="33"/>
+      <c r="D96" s="33"/>
+      <c r="E96" s="33"/>
+      <c r="F96" s="33"/>
+      <c r="G96" s="33"/>
+      <c r="H96" s="39"/>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A97" s="49"/>
+      <c r="B97" s="35"/>
+      <c r="C97" s="35"/>
+      <c r="D97" s="35"/>
+      <c r="E97" s="35"/>
+      <c r="F97" s="35"/>
+      <c r="G97" s="35"/>
+      <c r="H97" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A96:H97"/>
+    <mergeCell ref="B91:H91"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="B90:H90"/>
+    <mergeCell ref="A84:H84"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="B93:H93"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="B86:H86"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="C6:H6"/>
     <mergeCell ref="A20:E20"/>
+    <mergeCell ref="B88:H88"/>
     <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="B87:H87"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="B89:H89"/>
     <mergeCell ref="B85:H85"/>
-    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="B94:H94"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="B81:H81"/>
     <mergeCell ref="C7:H7"/>
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B86:H86"/>
-    <mergeCell ref="B84:H84"/>
-    <mergeCell ref="B83:H83"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A83:H83"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A80:F80"/>
     <mergeCell ref="C9:H9"/>
-    <mergeCell ref="A75:F75"/>
-    <mergeCell ref="A91:H92"/>
+    <mergeCell ref="B92:H92"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="B88:H88"/>
-    <mergeCell ref="B82:H82"/>
-    <mergeCell ref="B87:H87"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
docs: add demo videos, fix architecture heading, rename tech stack section
</commit_message>
<xml_diff>
--- a/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
+++ b/QuotationSheet/Delhi_PS_CRM_Quotation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Delhi-PS-CRM\QuotationSheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4354CD33-15F4-43BC-A25B-4BD6D11086FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90091F33-5AA0-4D85-81E7-CAFA9AEEB490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3768" yWindow="3768" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quotation" sheetId="1" r:id="rId1"/>
@@ -797,7 +797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -869,72 +869,78 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1250,118 +1256,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="31"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="50" t="s">
+      <c r="B6" s="30"/>
+      <c r="C6" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="39"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="31"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="50" t="s">
+      <c r="B7" s="30"/>
+      <c r="C7" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="39"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="31"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="50" t="s">
+      <c r="B8" s="30"/>
+      <c r="C8" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="39"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="31"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="55" t="s">
+      <c r="A9" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="36" t="s">
+      <c r="B9" s="33"/>
+      <c r="C9" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="37"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="34"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="31"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="45"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -1492,39 +1498,39 @@
       <c r="A19" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
       <c r="F19" s="12">
         <f>G31+G40+G53+G66</f>
         <v>263958</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="55" t="s">
+      <c r="A20" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
       <c r="F20" s="13">
         <f>G80*12</f>
         <v>706680</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="31"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="45"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
@@ -1742,14 +1748,14 @@
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
+      <c r="B31" s="30"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
       <c r="G31" s="20">
         <f>SUM(G24:G30)</f>
         <v>60750</v>
@@ -1973,14 +1979,14 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40" s="32" t="s">
+      <c r="A40" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="B40" s="33"/>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="30"/>
+      <c r="D40" s="30"/>
+      <c r="E40" s="30"/>
+      <c r="F40" s="30"/>
       <c r="G40" s="20">
         <f>SUM(G32:G39)</f>
         <v>51250</v>
@@ -2312,14 +2318,14 @@
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="32" t="s">
+      <c r="A53" s="41" t="s">
         <v>127</v>
       </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="33"/>
-      <c r="D53" s="33"/>
-      <c r="E53" s="33"/>
-      <c r="F53" s="33"/>
+      <c r="B53" s="30"/>
+      <c r="C53" s="30"/>
+      <c r="D53" s="30"/>
+      <c r="E53" s="30"/>
+      <c r="F53" s="30"/>
       <c r="G53" s="20">
         <f>SUM(G41:G52)</f>
         <v>68588</v>
@@ -2651,14 +2657,14 @@
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A66" s="32" t="s">
+      <c r="A66" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="B66" s="33"/>
-      <c r="C66" s="33"/>
-      <c r="D66" s="33"/>
-      <c r="E66" s="33"/>
-      <c r="F66" s="33"/>
+      <c r="B66" s="30"/>
+      <c r="C66" s="30"/>
+      <c r="D66" s="30"/>
+      <c r="E66" s="30"/>
+      <c r="F66" s="30"/>
       <c r="G66" s="20">
         <f>SUM(G54:G65)</f>
         <v>83370</v>
@@ -3017,14 +3023,14 @@
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A80" s="34" t="s">
+      <c r="A80" s="55" t="s">
         <v>156</v>
       </c>
-      <c r="B80" s="35"/>
-      <c r="C80" s="35"/>
-      <c r="D80" s="35"/>
-      <c r="E80" s="35"/>
-      <c r="F80" s="35"/>
+      <c r="B80" s="33"/>
+      <c r="C80" s="33"/>
+      <c r="D80" s="33"/>
+      <c r="E80" s="33"/>
+      <c r="F80" s="33"/>
       <c r="G80" s="22">
         <f>SUM(G67:G79)</f>
         <v>58890</v>
@@ -3032,173 +3038,173 @@
       <c r="H80" s="23"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A83" s="29" t="s">
+      <c r="A83" s="43" t="s">
         <v>157</v>
       </c>
-      <c r="B83" s="30"/>
-      <c r="C83" s="30"/>
-      <c r="D83" s="30"/>
-      <c r="E83" s="30"/>
-      <c r="F83" s="30"/>
-      <c r="G83" s="30"/>
-      <c r="H83" s="31"/>
+      <c r="B83" s="44"/>
+      <c r="C83" s="44"/>
+      <c r="D83" s="44"/>
+      <c r="E83" s="44"/>
+      <c r="F83" s="44"/>
+      <c r="G83" s="44"/>
+      <c r="H83" s="45"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A84" s="51" t="s">
+      <c r="A84" s="40" t="s">
         <v>158</v>
       </c>
-      <c r="B84" s="33"/>
-      <c r="C84" s="33"/>
-      <c r="D84" s="33"/>
-      <c r="E84" s="33"/>
-      <c r="F84" s="33"/>
-      <c r="G84" s="33"/>
-      <c r="H84" s="39"/>
+      <c r="B84" s="30"/>
+      <c r="C84" s="30"/>
+      <c r="D84" s="30"/>
+      <c r="E84" s="30"/>
+      <c r="F84" s="30"/>
+      <c r="G84" s="30"/>
+      <c r="H84" s="31"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B85" s="46" t="s">
+      <c r="B85" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="C85" s="46"/>
-      <c r="D85" s="46"/>
-      <c r="E85" s="46"/>
-      <c r="F85" s="46"/>
-      <c r="G85" s="46"/>
-      <c r="H85" s="47"/>
+      <c r="C85" s="51"/>
+      <c r="D85" s="51"/>
+      <c r="E85" s="51"/>
+      <c r="F85" s="51"/>
+      <c r="G85" s="51"/>
+      <c r="H85" s="52"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="B86" s="38">
+      <c r="B86" s="39">
         <f>G31+G40+G53+G66</f>
         <v>263958</v>
       </c>
-      <c r="C86" s="33"/>
-      <c r="D86" s="33"/>
-      <c r="E86" s="33"/>
-      <c r="F86" s="33"/>
-      <c r="G86" s="33"/>
-      <c r="H86" s="39"/>
+      <c r="C86" s="30"/>
+      <c r="D86" s="30"/>
+      <c r="E86" s="30"/>
+      <c r="F86" s="30"/>
+      <c r="G86" s="30"/>
+      <c r="H86" s="31"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="B87" s="57">
+      <c r="B87" s="48">
         <f>G80*12</f>
         <v>706680</v>
       </c>
-      <c r="C87" s="44"/>
-      <c r="D87" s="44"/>
-      <c r="E87" s="44"/>
-      <c r="F87" s="44"/>
-      <c r="G87" s="44"/>
-      <c r="H87" s="45"/>
+      <c r="C87" s="36"/>
+      <c r="D87" s="36"/>
+      <c r="E87" s="36"/>
+      <c r="F87" s="36"/>
+      <c r="G87" s="36"/>
+      <c r="H87" s="37"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="B88" s="56">
+      <c r="B88" s="47">
         <f>G80/272</f>
         <v>216.50735294117646</v>
       </c>
-      <c r="C88" s="33"/>
-      <c r="D88" s="33"/>
-      <c r="E88" s="33"/>
-      <c r="F88" s="33"/>
-      <c r="G88" s="33"/>
-      <c r="H88" s="39"/>
+      <c r="C88" s="30"/>
+      <c r="D88" s="30"/>
+      <c r="E88" s="30"/>
+      <c r="F88" s="30"/>
+      <c r="G88" s="30"/>
+      <c r="H88" s="31"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="B89" s="43">
+      <c r="B89" s="35">
         <f>G80/100000</f>
         <v>0.58889999999999998</v>
       </c>
-      <c r="C89" s="44"/>
-      <c r="D89" s="44"/>
-      <c r="E89" s="44"/>
-      <c r="F89" s="44"/>
-      <c r="G89" s="44"/>
-      <c r="H89" s="45"/>
+      <c r="C89" s="36"/>
+      <c r="D89" s="36"/>
+      <c r="E89" s="36"/>
+      <c r="F89" s="36"/>
+      <c r="G89" s="36"/>
+      <c r="H89" s="37"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="B90" s="38">
+      <c r="B90" s="39">
         <v>200000000</v>
       </c>
-      <c r="C90" s="33"/>
-      <c r="D90" s="33"/>
-      <c r="E90" s="33"/>
-      <c r="F90" s="33"/>
-      <c r="G90" s="33"/>
-      <c r="H90" s="39"/>
+      <c r="C90" s="30"/>
+      <c r="D90" s="30"/>
+      <c r="E90" s="30"/>
+      <c r="F90" s="30"/>
+      <c r="G90" s="30"/>
+      <c r="H90" s="31"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="B91" s="43">
+      <c r="B91" s="35">
         <f>G80*12/200000000</f>
         <v>3.5333999999999999E-3</v>
       </c>
-      <c r="C91" s="44"/>
-      <c r="D91" s="44"/>
-      <c r="E91" s="44"/>
-      <c r="F91" s="44"/>
-      <c r="G91" s="44"/>
-      <c r="H91" s="45"/>
+      <c r="C91" s="36"/>
+      <c r="D91" s="36"/>
+      <c r="E91" s="36"/>
+      <c r="F91" s="36"/>
+      <c r="G91" s="36"/>
+      <c r="H91" s="37"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="B92" s="38">
+      <c r="B92" s="39">
         <v>272</v>
       </c>
-      <c r="C92" s="33"/>
-      <c r="D92" s="33"/>
-      <c r="E92" s="33"/>
-      <c r="F92" s="33"/>
-      <c r="G92" s="33"/>
-      <c r="H92" s="39"/>
+      <c r="C92" s="30"/>
+      <c r="D92" s="30"/>
+      <c r="E92" s="30"/>
+      <c r="F92" s="30"/>
+      <c r="G92" s="30"/>
+      <c r="H92" s="31"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="B93" s="53" t="s">
+      <c r="B93" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="C93" s="44"/>
-      <c r="D93" s="44"/>
-      <c r="E93" s="44"/>
-      <c r="F93" s="44"/>
-      <c r="G93" s="44"/>
-      <c r="H93" s="45"/>
+      <c r="C93" s="58"/>
+      <c r="D93" s="58"/>
+      <c r="E93" s="58"/>
+      <c r="F93" s="58"/>
+      <c r="G93" s="58"/>
+      <c r="H93" s="59"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="B94" s="38">
+      <c r="B94" s="39">
         <v>1200000</v>
       </c>
-      <c r="C94" s="33"/>
-      <c r="D94" s="33"/>
-      <c r="E94" s="33"/>
-      <c r="F94" s="33"/>
-      <c r="G94" s="33"/>
-      <c r="H94" s="39"/>
+      <c r="C94" s="30"/>
+      <c r="D94" s="30"/>
+      <c r="E94" s="30"/>
+      <c r="F94" s="30"/>
+      <c r="G94" s="30"/>
+      <c r="H94" s="31"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="26"/>
@@ -3211,29 +3217,47 @@
       <c r="H95" s="28"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A96" s="48" t="s">
+      <c r="A96" s="29" t="s">
         <v>170</v>
       </c>
-      <c r="B96" s="33"/>
-      <c r="C96" s="33"/>
-      <c r="D96" s="33"/>
-      <c r="E96" s="33"/>
-      <c r="F96" s="33"/>
-      <c r="G96" s="33"/>
-      <c r="H96" s="39"/>
+      <c r="B96" s="30"/>
+      <c r="C96" s="30"/>
+      <c r="D96" s="30"/>
+      <c r="E96" s="30"/>
+      <c r="F96" s="30"/>
+      <c r="G96" s="30"/>
+      <c r="H96" s="31"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A97" s="49"/>
-      <c r="B97" s="35"/>
-      <c r="C97" s="35"/>
-      <c r="D97" s="35"/>
-      <c r="E97" s="35"/>
-      <c r="F97" s="35"/>
-      <c r="G97" s="35"/>
-      <c r="H97" s="37"/>
+      <c r="A97" s="32"/>
+      <c r="B97" s="33"/>
+      <c r="C97" s="33"/>
+      <c r="D97" s="33"/>
+      <c r="E97" s="33"/>
+      <c r="F97" s="33"/>
+      <c r="G97" s="33"/>
+      <c r="H97" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="B92:H92"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="B89:H89"/>
+    <mergeCell ref="B85:H85"/>
+    <mergeCell ref="B94:H94"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A83:H83"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="C9:H9"/>
     <mergeCell ref="A96:H97"/>
     <mergeCell ref="B91:H91"/>
     <mergeCell ref="C8:H8"/>
@@ -3250,24 +3274,6 @@
     <mergeCell ref="B88:H88"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="B87:H87"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="B89:H89"/>
-    <mergeCell ref="B85:H85"/>
-    <mergeCell ref="B94:H94"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A83:H83"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A80:F80"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="B92:H92"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>

</xml_diff>